<commit_message>
Rate/inflation sensitivity grid in the style of the WACC-vs-g heatmap (target price per cell, base highlighted); Excel block E
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0188QZHBkA8n5QL7BtmFakQg
</commit_message>
<xml_diff>
--- a/secciones/valuacion/modelos/Mallplaza_Sensibilidad_Tasas_Inflacion.xlsx
+++ b/secciones/valuacion/modelos/Mallplaza_Sensibilidad_Tasas_Inflacion.xlsx
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="225" uniqueCount="131">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="227" uniqueCount="133">
   <si>
     <t xml:space="preserve">Sensibilidad del valor por acción a tasas largas e inflación (NUEVO)</t>
   </si>
@@ -89,6 +89,12 @@
   </si>
   <si>
     <t xml:space="preserve">Lectura: el DCF dice que una alza de 100 pb de tasa real baja el valor ~17%, mientras que la inflación casi no lo mueve; en el dato histórico la sensibilidad es mucho menor y poco significativa porque la acción se re-valorizó con tasas casi planas.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">E. Precio objetivo (80% DCF + 20% múltiplos, múltiplos fijos): filas = inflación esperada, columnas = tasa real a 10 años (BCU10, base 30-09-26)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tasa real / inflación</t>
   </si>
   <si>
     <t xml:space="preserve">Sensibilidad a tasas largas e inflación — insumos</t>
@@ -422,9 +428,10 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="2">
+  <numFmts count="3">
     <numFmt numFmtId="164" formatCode="General"/>
-    <numFmt numFmtId="165" formatCode="dd\-mm\-yyyy"/>
+    <numFmt numFmtId="165" formatCode="General"/>
+    <numFmt numFmtId="166" formatCode="dd\-mm\-yyyy"/>
   </numFmts>
   <fonts count="6">
     <font>
@@ -512,7 +519,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="8">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -525,11 +532,15 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -537,7 +548,7 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="166" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -733,7 +744,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:L37"/>
+  <dimension ref="A1:L46"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1545,6 +1556,166 @@
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="0" t="s">
         <v>21</v>
+      </c>
+    </row>
+    <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A40" s="3" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A41" s="0" t="s">
+        <v>23</v>
+      </c>
+      <c r="B41" s="0" t="n">
+        <f aca="false">2.82/100+-100/10000</f>
+        <v>0.0182</v>
+      </c>
+      <c r="C41" s="0" t="n">
+        <f aca="false">2.82/100+-50/10000</f>
+        <v>0.0232</v>
+      </c>
+      <c r="D41" s="0" t="n">
+        <f aca="false">2.82/100+0/10000</f>
+        <v>0.0282</v>
+      </c>
+      <c r="E41" s="0" t="n">
+        <f aca="false">2.82/100+50/10000</f>
+        <v>0.0332</v>
+      </c>
+      <c r="F41" s="0" t="n">
+        <f aca="false">2.82/100+100/10000</f>
+        <v>0.0382</v>
+      </c>
+    </row>
+    <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A42" s="0" t="n">
+        <f aca="false">Supuestos!$B$4+100/10000</f>
+        <v>0.04</v>
+      </c>
+      <c r="B42" s="0" t="n">
+        <f aca="false">Supuestos!$B$12*Calculo!AI35+(1-Supuestos!$B$12)*Supuestos!$B$11</f>
+        <v>2396.37158617503</v>
+      </c>
+      <c r="C42" s="0" t="n">
+        <f aca="false">Supuestos!$B$12*Calculo!AI36+(1-Supuestos!$B$12)*Supuestos!$B$11</f>
+        <v>2221.47215684732</v>
+      </c>
+      <c r="D42" s="0" t="n">
+        <f aca="false">Supuestos!$B$12*Calculo!AI37+(1-Supuestos!$B$12)*Supuestos!$B$11</f>
+        <v>2069.99520538708</v>
+      </c>
+      <c r="E42" s="0" t="n">
+        <f aca="false">Supuestos!$B$12*Calculo!AI38+(1-Supuestos!$B$12)*Supuestos!$B$11</f>
+        <v>1937.58878276197</v>
+      </c>
+      <c r="F42" s="0" t="n">
+        <f aca="false">Supuestos!$B$12*Calculo!AI39+(1-Supuestos!$B$12)*Supuestos!$B$11</f>
+        <v>1820.9138255286</v>
+      </c>
+    </row>
+    <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A43" s="0" t="n">
+        <f aca="false">Supuestos!$B$4+50/10000</f>
+        <v>0.035</v>
+      </c>
+      <c r="B43" s="0" t="n">
+        <f aca="false">Supuestos!$B$12*Calculo!AI28+(1-Supuestos!$B$12)*Supuestos!$B$11</f>
+        <v>2398.52282169555</v>
+      </c>
+      <c r="C43" s="0" t="n">
+        <f aca="false">Supuestos!$B$12*Calculo!AI29+(1-Supuestos!$B$12)*Supuestos!$B$11</f>
+        <v>2224.00504632591</v>
+      </c>
+      <c r="D43" s="0" t="n">
+        <f aca="false">Supuestos!$B$12*Calculo!AI30+(1-Supuestos!$B$12)*Supuestos!$B$11</f>
+        <v>2072.77343294611</v>
+      </c>
+      <c r="E43" s="0" t="n">
+        <f aca="false">Supuestos!$B$12*Calculo!AI31+(1-Supuestos!$B$12)*Supuestos!$B$11</f>
+        <v>1940.51691298762</v>
+      </c>
+      <c r="F43" s="0" t="n">
+        <f aca="false">Supuestos!$B$12*Calculo!AI32+(1-Supuestos!$B$12)*Supuestos!$B$11</f>
+        <v>1823.92435425508</v>
+      </c>
+    </row>
+    <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A44" s="0" t="n">
+        <f aca="false">Supuestos!$B$4+0/10000</f>
+        <v>0.03</v>
+      </c>
+      <c r="B44" s="0" t="n">
+        <f aca="false">Supuestos!$B$12*Calculo!AI21+(1-Supuestos!$B$12)*Supuestos!$B$11</f>
+        <v>2400.87840988789</v>
+      </c>
+      <c r="C44" s="0" t="n">
+        <f aca="false">Supuestos!$B$12*Calculo!AI22+(1-Supuestos!$B$12)*Supuestos!$B$11</f>
+        <v>2226.72643573829</v>
+      </c>
+      <c r="D44" s="3" t="n">
+        <f aca="false">Supuestos!$B$12*Calculo!AI23+(1-Supuestos!$B$12)*Supuestos!$B$11</f>
+        <v>2075.72669191032</v>
+      </c>
+      <c r="E44" s="4" t="n">
+        <f aca="false">Supuestos!$B$12*Calculo!AI24+(1-Supuestos!$B$12)*Supuestos!$B$11</f>
+        <v>1943.60840185851</v>
+      </c>
+      <c r="F44" s="4" t="n">
+        <f aca="false">Supuestos!$B$12*Calculo!AI25+(1-Supuestos!$B$12)*Supuestos!$B$11</f>
+        <v>1827.08796807026</v>
+      </c>
+    </row>
+    <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A45" s="0" t="n">
+        <f aca="false">Supuestos!$B$4+-50/10000</f>
+        <v>0.025</v>
+      </c>
+      <c r="B45" s="0" t="n">
+        <f aca="false">Supuestos!$B$12*Calculo!AI14+(1-Supuestos!$B$12)*Supuestos!$B$11</f>
+        <v>2403.44603891151</v>
+      </c>
+      <c r="C45" s="0" t="n">
+        <f aca="false">Supuestos!$B$12*Calculo!AI15+(1-Supuestos!$B$12)*Supuestos!$B$11</f>
+        <v>2229.64351386822</v>
+      </c>
+      <c r="D45" s="0" t="n">
+        <f aca="false">Supuestos!$B$12*Calculo!AI16+(1-Supuestos!$B$12)*Supuestos!$B$11</f>
+        <v>2078.86171657788</v>
+      </c>
+      <c r="E45" s="0" t="n">
+        <f aca="false">Supuestos!$B$12*Calculo!AI17+(1-Supuestos!$B$12)*Supuestos!$B$11</f>
+        <v>1946.86957007491</v>
+      </c>
+      <c r="F45" s="0" t="n">
+        <f aca="false">Supuestos!$B$12*Calculo!AI18+(1-Supuestos!$B$12)*Supuestos!$B$11</f>
+        <v>1830.41061070193</v>
+      </c>
+    </row>
+    <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A46" s="0" t="n">
+        <f aca="false">Supuestos!$B$4+-100/10000</f>
+        <v>0.02</v>
+      </c>
+      <c r="B46" s="0" t="n">
+        <f aca="false">Supuestos!$B$12*Calculo!AI7+(1-Supuestos!$B$12)*Supuestos!$B$11</f>
+        <v>2406.23370717642</v>
+      </c>
+      <c r="C46" s="0" t="n">
+        <f aca="false">Supuestos!$B$12*Calculo!AI8+(1-Supuestos!$B$12)*Supuestos!$B$11</f>
+        <v>2232.76376155139</v>
+      </c>
+      <c r="D46" s="0" t="n">
+        <f aca="false">Supuestos!$B$12*Calculo!AI9+(1-Supuestos!$B$12)*Supuestos!$B$11</f>
+        <v>2082.18551649992</v>
+      </c>
+      <c r="E46" s="0" t="n">
+        <f aca="false">Supuestos!$B$12*Calculo!AI10+(1-Supuestos!$B$12)*Supuestos!$B$11</f>
+        <v>1950.30699807294</v>
+      </c>
+      <c r="F46" s="0" t="n">
+        <f aca="false">Supuestos!$B$12*Calculo!AI11+(1-Supuestos!$B$12)*Supuestos!$B$11</f>
+        <v>1833.8984712684</v>
       </c>
     </row>
   </sheetData>
@@ -1568,160 +1739,160 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="0" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="0" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="0" t="s">
-        <v>24</v>
-      </c>
-      <c r="B4" s="3" t="n">
+        <v>26</v>
+      </c>
+      <c r="B4" s="5" t="n">
         <v>0.03</v>
       </c>
       <c r="K4" s="4" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="0" t="s">
-        <v>26</v>
-      </c>
-      <c r="B5" s="3" t="n">
+        <v>28</v>
+      </c>
+      <c r="B5" s="5" t="n">
         <v>0.03</v>
       </c>
       <c r="K5" s="4" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="0" t="s">
-        <v>28</v>
-      </c>
-      <c r="B6" s="3" t="n">
+        <v>30</v>
+      </c>
+      <c r="B6" s="5" t="n">
         <v>0.27</v>
       </c>
       <c r="K6" s="4" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="0" t="s">
-        <v>30</v>
-      </c>
-      <c r="B7" s="3" t="n">
+        <v>32</v>
+      </c>
+      <c r="B7" s="5" t="n">
         <v>1285740</v>
       </c>
       <c r="K7" s="4" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="0" t="s">
-        <v>32</v>
-      </c>
-      <c r="B8" s="3" t="n">
+        <v>34</v>
+      </c>
+      <c r="B8" s="5" t="n">
         <v>50841</v>
       </c>
       <c r="K8" s="4" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="0" t="s">
-        <v>34</v>
-      </c>
-      <c r="B9" s="3" t="n">
+        <v>36</v>
+      </c>
+      <c r="B9" s="5" t="n">
         <v>2190</v>
       </c>
       <c r="K9" s="4" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="0" t="s">
-        <v>36</v>
-      </c>
-      <c r="B10" s="3" t="n">
+        <v>38</v>
+      </c>
+      <c r="B10" s="5" t="n">
         <v>3555</v>
       </c>
       <c r="K10" s="4" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="0" t="s">
-        <v>38</v>
-      </c>
-      <c r="B11" s="3" t="n">
+        <v>40</v>
+      </c>
+      <c r="B11" s="5" t="n">
         <v>2951.38547083101</v>
       </c>
       <c r="K11" s="4" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="0" t="s">
-        <v>40</v>
-      </c>
-      <c r="B12" s="3" t="n">
+        <v>42</v>
+      </c>
+      <c r="B12" s="5" t="n">
         <v>0.8</v>
       </c>
       <c r="K12" s="4" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="0" t="s">
-        <v>42</v>
-      </c>
-      <c r="B13" s="5" t="n">
+        <v>44</v>
+      </c>
+      <c r="B13" s="6" t="n">
         <v>0.85</v>
       </c>
       <c r="K13" s="4" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="0" t="s">
-        <v>44</v>
-      </c>
-      <c r="B14" s="5" t="n">
+        <v>46</v>
+      </c>
+      <c r="B14" s="6" t="n">
         <v>1</v>
       </c>
       <c r="K14" s="4" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="0" t="s">
-        <v>46</v>
-      </c>
-      <c r="B15" s="3" t="n">
+        <v>48</v>
+      </c>
+      <c r="B15" s="5" t="n">
         <v>100</v>
       </c>
       <c r="K15" s="4" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="0" t="s">
-        <v>48</v>
-      </c>
-      <c r="B16" s="3" t="n">
+        <v>50</v>
+      </c>
+      <c r="B16" s="5" t="n">
         <v>0</v>
       </c>
       <c r="K16" s="4" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="0" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="B19" s="0" t="n">
         <f aca="false">Calculo!AI107</f>
@@ -1730,7 +1901,7 @@
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="0" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="B20" s="0" t="n">
         <f aca="false">B19/Calculo!AI5-1</f>
@@ -1739,199 +1910,199 @@
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="0" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="C22" s="0" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="D22" s="0" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="E22" s="0" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="F22" s="0" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="G22" s="0" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="H22" s="0" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="I22" s="0" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="0" t="s">
-        <v>60</v>
-      </c>
-      <c r="C23" s="3" t="n">
+        <v>62</v>
+      </c>
+      <c r="C23" s="5" t="n">
         <v>113425.715768245</v>
       </c>
-      <c r="D23" s="3" t="n">
+      <c r="D23" s="5" t="n">
         <v>199440.442268561</v>
       </c>
-      <c r="E23" s="3" t="n">
+      <c r="E23" s="5" t="n">
         <v>259687.719258378</v>
       </c>
-      <c r="F23" s="3" t="n">
+      <c r="F23" s="5" t="n">
         <v>375320.615932717</v>
       </c>
-      <c r="G23" s="3" t="n">
+      <c r="G23" s="5" t="n">
         <v>377068.219372121</v>
       </c>
-      <c r="H23" s="3" t="n">
+      <c r="H23" s="5" t="n">
         <v>398715.503513791</v>
       </c>
-      <c r="I23" s="3" t="n">
+      <c r="I23" s="5" t="n">
         <v>528835.311960595</v>
       </c>
       <c r="K23" s="4" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="0" t="s">
-        <v>62</v>
-      </c>
-      <c r="C24" s="3" t="n">
+        <v>64</v>
+      </c>
+      <c r="C24" s="5" t="n">
         <v>0.5</v>
       </c>
-      <c r="D24" s="3" t="n">
+      <c r="D24" s="5" t="n">
         <v>1</v>
       </c>
-      <c r="E24" s="3" t="n">
+      <c r="E24" s="5" t="n">
         <v>1</v>
       </c>
-      <c r="F24" s="3" t="n">
+      <c r="F24" s="5" t="n">
         <v>1</v>
       </c>
-      <c r="G24" s="3" t="n">
+      <c r="G24" s="5" t="n">
         <v>1</v>
       </c>
-      <c r="H24" s="3" t="n">
+      <c r="H24" s="5" t="n">
         <v>1</v>
       </c>
       <c r="K24" s="4" t="s">
-        <v>63</v>
+        <v>65</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="0" t="s">
-        <v>64</v>
-      </c>
-      <c r="C25" s="3" t="n">
+        <v>66</v>
+      </c>
+      <c r="C25" s="5" t="n">
         <v>0.25</v>
       </c>
-      <c r="D25" s="3" t="n">
+      <c r="D25" s="5" t="n">
         <v>1</v>
       </c>
-      <c r="E25" s="3" t="n">
+      <c r="E25" s="5" t="n">
         <v>2</v>
       </c>
-      <c r="F25" s="3" t="n">
+      <c r="F25" s="5" t="n">
         <v>3</v>
       </c>
-      <c r="G25" s="3" t="n">
+      <c r="G25" s="5" t="n">
         <v>4</v>
       </c>
-      <c r="H25" s="3" t="n">
+      <c r="H25" s="5" t="n">
         <v>5</v>
       </c>
-      <c r="I25" s="3" t="n">
+      <c r="I25" s="5" t="n">
         <v>6</v>
       </c>
       <c r="K25" s="4" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="0" t="s">
-        <v>66</v>
-      </c>
-      <c r="C26" s="3" t="n">
+        <v>68</v>
+      </c>
+      <c r="C26" s="5" t="n">
         <v>0.117033041180547</v>
       </c>
-      <c r="D26" s="3" t="n">
+      <c r="D26" s="5" t="n">
         <v>0.117479013178444</v>
       </c>
-      <c r="E26" s="3" t="n">
+      <c r="E26" s="5" t="n">
         <v>0.11792498517634</v>
       </c>
-      <c r="F26" s="3" t="n">
+      <c r="F26" s="5" t="n">
         <v>0.118370957174237</v>
       </c>
-      <c r="G26" s="3" t="n">
+      <c r="G26" s="5" t="n">
         <v>0.118816929172134</v>
       </c>
-      <c r="H26" s="3" t="n">
+      <c r="H26" s="5" t="n">
         <v>0.119262901170031</v>
       </c>
-      <c r="I26" s="3" t="n">
+      <c r="I26" s="5" t="n">
         <v>0.119262901170031</v>
       </c>
       <c r="K26" s="4" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="0" t="s">
-        <v>68</v>
-      </c>
-      <c r="C27" s="3" t="n">
+        <v>70</v>
+      </c>
+      <c r="C27" s="5" t="n">
         <v>0.0362592187808888</v>
       </c>
-      <c r="D27" s="3" t="n">
+      <c r="D27" s="5" t="n">
         <v>0.0367776563426664</v>
       </c>
-      <c r="E27" s="3" t="n">
+      <c r="E27" s="5" t="n">
         <v>0.037296093904444</v>
       </c>
-      <c r="F27" s="3" t="n">
+      <c r="F27" s="5" t="n">
         <v>0.0378145314662216</v>
       </c>
-      <c r="G27" s="3" t="n">
+      <c r="G27" s="5" t="n">
         <v>0.0383329690279992</v>
       </c>
-      <c r="H27" s="3" t="n">
+      <c r="H27" s="5" t="n">
         <v>0.0388514065897768</v>
       </c>
-      <c r="I27" s="3" t="n">
+      <c r="I27" s="5" t="n">
         <v>0.0388514065897768</v>
       </c>
       <c r="K27" s="4" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="0" t="s">
-        <v>70</v>
-      </c>
-      <c r="C28" s="3" t="n">
+        <v>72</v>
+      </c>
+      <c r="C28" s="5" t="n">
         <v>0.171864958306498</v>
       </c>
-      <c r="D28" s="3" t="n">
+      <c r="D28" s="5" t="n">
         <v>0.182384862157361</v>
       </c>
-      <c r="E28" s="3" t="n">
+      <c r="E28" s="5" t="n">
         <v>0.192640847271158</v>
       </c>
-      <c r="F28" s="3" t="n">
+      <c r="F28" s="5" t="n">
         <v>0.202642722227619</v>
       </c>
-      <c r="G28" s="3" t="n">
+      <c r="G28" s="5" t="n">
         <v>0.212399815504365</v>
       </c>
-      <c r="H28" s="3" t="n">
+      <c r="H28" s="5" t="n">
         <v>0.221921004496352</v>
       </c>
-      <c r="I28" s="3" t="n">
+      <c r="I28" s="5" t="n">
         <v>0.221921004496352</v>
       </c>
       <c r="K28" s="4" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
     </row>
   </sheetData>
@@ -1955,122 +2126,122 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="0" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="0" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="0" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="B4" s="0" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="C4" s="0" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="D4" s="0" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="E4" s="0" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="F4" s="0" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="G4" s="0" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="H4" s="0" t="s">
-        <v>81</v>
+        <v>83</v>
       </c>
       <c r="I4" s="0" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="J4" s="0" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="K4" s="0" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="L4" s="0" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="M4" s="0" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="N4" s="0" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="O4" s="0" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="P4" s="0" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="Q4" s="0" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="R4" s="0" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="S4" s="0" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="T4" s="0" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="U4" s="0" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="V4" s="0" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="W4" s="0" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="X4" s="0" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="Y4" s="0" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="Z4" s="0" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="AA4" s="0" t="s">
-        <v>100</v>
+        <v>102</v>
       </c>
       <c r="AB4" s="0" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
       <c r="AC4" s="0" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
       <c r="AD4" s="0" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="AE4" s="0" t="s">
-        <v>104</v>
+        <v>106</v>
       </c>
       <c r="AF4" s="0" t="s">
-        <v>105</v>
+        <v>107</v>
       </c>
       <c r="AG4" s="0" t="s">
-        <v>106</v>
+        <v>108</v>
       </c>
       <c r="AH4" s="0" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="AI4" s="0" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
       <c r="AJ4" s="0" t="s">
-        <v>109</v>
+        <v>111</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2085,7 +2256,7 @@
         <v>0.85</v>
       </c>
       <c r="D5" s="0" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="E5" s="0" t="n">
         <f aca="false">(1-Supuestos!C$28)*((1+((1+Supuestos!C$26)/(1+Supuestos!$B$4)-1+Supuestos!$B$14*$A5/10000))*(1+Supuestos!$B$4+$B5/10000)-1)+Supuestos!C$28*((1+Supuestos!C$27+$A5/10000)*(1+Supuestos!$B$4+$B5/10000)-1)*(1-Supuestos!$B$6)</f>
@@ -2228,7 +2399,7 @@
         <v>0.85</v>
       </c>
       <c r="D6" s="0" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="E6" s="0" t="n">
         <f aca="false">(1-Supuestos!C$28)*((1+((1+Supuestos!C$26)/(1+Supuestos!$B$4)-1+Supuestos!$B$14*$A6/10000))*(1+Supuestos!$B$4+$B6/10000)-1)+Supuestos!C$28*((1+Supuestos!C$27+$A6/10000)*(1+Supuestos!$B$4+$B6/10000)-1)*(1-Supuestos!$B$6)</f>
@@ -2371,7 +2542,7 @@
         <v>0.85</v>
       </c>
       <c r="D7" s="0" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="E7" s="0" t="n">
         <f aca="false">(1-Supuestos!C$28)*((1+((1+Supuestos!C$26)/(1+Supuestos!$B$4)-1+Supuestos!$B$14*$A7/10000))*(1+Supuestos!$B$4+$B7/10000)-1)+Supuestos!C$28*((1+Supuestos!C$27+$A7/10000)*(1+Supuestos!$B$4+$B7/10000)-1)*(1-Supuestos!$B$6)</f>
@@ -2514,7 +2685,7 @@
         <v>0.85</v>
       </c>
       <c r="D8" s="0" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="E8" s="0" t="n">
         <f aca="false">(1-Supuestos!C$28)*((1+((1+Supuestos!C$26)/(1+Supuestos!$B$4)-1+Supuestos!$B$14*$A8/10000))*(1+Supuestos!$B$4+$B8/10000)-1)+Supuestos!C$28*((1+Supuestos!C$27+$A8/10000)*(1+Supuestos!$B$4+$B8/10000)-1)*(1-Supuestos!$B$6)</f>
@@ -2657,7 +2828,7 @@
         <v>0.85</v>
       </c>
       <c r="D9" s="0" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="E9" s="0" t="n">
         <f aca="false">(1-Supuestos!C$28)*((1+((1+Supuestos!C$26)/(1+Supuestos!$B$4)-1+Supuestos!$B$14*$A9/10000))*(1+Supuestos!$B$4+$B9/10000)-1)+Supuestos!C$28*((1+Supuestos!C$27+$A9/10000)*(1+Supuestos!$B$4+$B9/10000)-1)*(1-Supuestos!$B$6)</f>
@@ -2800,7 +2971,7 @@
         <v>0.85</v>
       </c>
       <c r="D10" s="0" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="E10" s="0" t="n">
         <f aca="false">(1-Supuestos!C$28)*((1+((1+Supuestos!C$26)/(1+Supuestos!$B$4)-1+Supuestos!$B$14*$A10/10000))*(1+Supuestos!$B$4+$B10/10000)-1)+Supuestos!C$28*((1+Supuestos!C$27+$A10/10000)*(1+Supuestos!$B$4+$B10/10000)-1)*(1-Supuestos!$B$6)</f>
@@ -2943,7 +3114,7 @@
         <v>0.85</v>
       </c>
       <c r="D11" s="0" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="E11" s="0" t="n">
         <f aca="false">(1-Supuestos!C$28)*((1+((1+Supuestos!C$26)/(1+Supuestos!$B$4)-1+Supuestos!$B$14*$A11/10000))*(1+Supuestos!$B$4+$B11/10000)-1)+Supuestos!C$28*((1+Supuestos!C$27+$A11/10000)*(1+Supuestos!$B$4+$B11/10000)-1)*(1-Supuestos!$B$6)</f>
@@ -3086,7 +3257,7 @@
         <v>0.85</v>
       </c>
       <c r="D12" s="0" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="E12" s="0" t="n">
         <f aca="false">(1-Supuestos!C$28)*((1+((1+Supuestos!C$26)/(1+Supuestos!$B$4)-1+Supuestos!$B$14*$A12/10000))*(1+Supuestos!$B$4+$B12/10000)-1)+Supuestos!C$28*((1+Supuestos!C$27+$A12/10000)*(1+Supuestos!$B$4+$B12/10000)-1)*(1-Supuestos!$B$6)</f>
@@ -3229,7 +3400,7 @@
         <v>0.85</v>
       </c>
       <c r="D13" s="0" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="E13" s="0" t="n">
         <f aca="false">(1-Supuestos!C$28)*((1+((1+Supuestos!C$26)/(1+Supuestos!$B$4)-1+Supuestos!$B$14*$A13/10000))*(1+Supuestos!$B$4+$B13/10000)-1)+Supuestos!C$28*((1+Supuestos!C$27+$A13/10000)*(1+Supuestos!$B$4+$B13/10000)-1)*(1-Supuestos!$B$6)</f>
@@ -3372,7 +3543,7 @@
         <v>0.85</v>
       </c>
       <c r="D14" s="0" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="E14" s="0" t="n">
         <f aca="false">(1-Supuestos!C$28)*((1+((1+Supuestos!C$26)/(1+Supuestos!$B$4)-1+Supuestos!$B$14*$A14/10000))*(1+Supuestos!$B$4+$B14/10000)-1)+Supuestos!C$28*((1+Supuestos!C$27+$A14/10000)*(1+Supuestos!$B$4+$B14/10000)-1)*(1-Supuestos!$B$6)</f>
@@ -3515,7 +3686,7 @@
         <v>0.85</v>
       </c>
       <c r="D15" s="0" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="E15" s="0" t="n">
         <f aca="false">(1-Supuestos!C$28)*((1+((1+Supuestos!C$26)/(1+Supuestos!$B$4)-1+Supuestos!$B$14*$A15/10000))*(1+Supuestos!$B$4+$B15/10000)-1)+Supuestos!C$28*((1+Supuestos!C$27+$A15/10000)*(1+Supuestos!$B$4+$B15/10000)-1)*(1-Supuestos!$B$6)</f>
@@ -3658,7 +3829,7 @@
         <v>0.85</v>
       </c>
       <c r="D16" s="0" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="E16" s="0" t="n">
         <f aca="false">(1-Supuestos!C$28)*((1+((1+Supuestos!C$26)/(1+Supuestos!$B$4)-1+Supuestos!$B$14*$A16/10000))*(1+Supuestos!$B$4+$B16/10000)-1)+Supuestos!C$28*((1+Supuestos!C$27+$A16/10000)*(1+Supuestos!$B$4+$B16/10000)-1)*(1-Supuestos!$B$6)</f>
@@ -3801,7 +3972,7 @@
         <v>0.85</v>
       </c>
       <c r="D17" s="0" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="E17" s="0" t="n">
         <f aca="false">(1-Supuestos!C$28)*((1+((1+Supuestos!C$26)/(1+Supuestos!$B$4)-1+Supuestos!$B$14*$A17/10000))*(1+Supuestos!$B$4+$B17/10000)-1)+Supuestos!C$28*((1+Supuestos!C$27+$A17/10000)*(1+Supuestos!$B$4+$B17/10000)-1)*(1-Supuestos!$B$6)</f>
@@ -3944,7 +4115,7 @@
         <v>0.85</v>
       </c>
       <c r="D18" s="0" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="E18" s="0" t="n">
         <f aca="false">(1-Supuestos!C$28)*((1+((1+Supuestos!C$26)/(1+Supuestos!$B$4)-1+Supuestos!$B$14*$A18/10000))*(1+Supuestos!$B$4+$B18/10000)-1)+Supuestos!C$28*((1+Supuestos!C$27+$A18/10000)*(1+Supuestos!$B$4+$B18/10000)-1)*(1-Supuestos!$B$6)</f>
@@ -4087,7 +4258,7 @@
         <v>0.85</v>
       </c>
       <c r="D19" s="0" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="E19" s="0" t="n">
         <f aca="false">(1-Supuestos!C$28)*((1+((1+Supuestos!C$26)/(1+Supuestos!$B$4)-1+Supuestos!$B$14*$A19/10000))*(1+Supuestos!$B$4+$B19/10000)-1)+Supuestos!C$28*((1+Supuestos!C$27+$A19/10000)*(1+Supuestos!$B$4+$B19/10000)-1)*(1-Supuestos!$B$6)</f>
@@ -4230,7 +4401,7 @@
         <v>0.85</v>
       </c>
       <c r="D20" s="0" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="E20" s="0" t="n">
         <f aca="false">(1-Supuestos!C$28)*((1+((1+Supuestos!C$26)/(1+Supuestos!$B$4)-1+Supuestos!$B$14*$A20/10000))*(1+Supuestos!$B$4+$B20/10000)-1)+Supuestos!C$28*((1+Supuestos!C$27+$A20/10000)*(1+Supuestos!$B$4+$B20/10000)-1)*(1-Supuestos!$B$6)</f>
@@ -4373,7 +4544,7 @@
         <v>0.85</v>
       </c>
       <c r="D21" s="0" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="E21" s="0" t="n">
         <f aca="false">(1-Supuestos!C$28)*((1+((1+Supuestos!C$26)/(1+Supuestos!$B$4)-1+Supuestos!$B$14*$A21/10000))*(1+Supuestos!$B$4+$B21/10000)-1)+Supuestos!C$28*((1+Supuestos!C$27+$A21/10000)*(1+Supuestos!$B$4+$B21/10000)-1)*(1-Supuestos!$B$6)</f>
@@ -4516,7 +4687,7 @@
         <v>0.85</v>
       </c>
       <c r="D22" s="0" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="E22" s="0" t="n">
         <f aca="false">(1-Supuestos!C$28)*((1+((1+Supuestos!C$26)/(1+Supuestos!$B$4)-1+Supuestos!$B$14*$A22/10000))*(1+Supuestos!$B$4+$B22/10000)-1)+Supuestos!C$28*((1+Supuestos!C$27+$A22/10000)*(1+Supuestos!$B$4+$B22/10000)-1)*(1-Supuestos!$B$6)</f>
@@ -4659,7 +4830,7 @@
         <v>0.85</v>
       </c>
       <c r="D23" s="0" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="E23" s="0" t="n">
         <f aca="false">(1-Supuestos!C$28)*((1+((1+Supuestos!C$26)/(1+Supuestos!$B$4)-1+Supuestos!$B$14*$A23/10000))*(1+Supuestos!$B$4+$B23/10000)-1)+Supuestos!C$28*((1+Supuestos!C$27+$A23/10000)*(1+Supuestos!$B$4+$B23/10000)-1)*(1-Supuestos!$B$6)</f>
@@ -4802,7 +4973,7 @@
         <v>0.85</v>
       </c>
       <c r="D24" s="0" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="E24" s="0" t="n">
         <f aca="false">(1-Supuestos!C$28)*((1+((1+Supuestos!C$26)/(1+Supuestos!$B$4)-1+Supuestos!$B$14*$A24/10000))*(1+Supuestos!$B$4+$B24/10000)-1)+Supuestos!C$28*((1+Supuestos!C$27+$A24/10000)*(1+Supuestos!$B$4+$B24/10000)-1)*(1-Supuestos!$B$6)</f>
@@ -4945,7 +5116,7 @@
         <v>0.85</v>
       </c>
       <c r="D25" s="0" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="E25" s="0" t="n">
         <f aca="false">(1-Supuestos!C$28)*((1+((1+Supuestos!C$26)/(1+Supuestos!$B$4)-1+Supuestos!$B$14*$A25/10000))*(1+Supuestos!$B$4+$B25/10000)-1)+Supuestos!C$28*((1+Supuestos!C$27+$A25/10000)*(1+Supuestos!$B$4+$B25/10000)-1)*(1-Supuestos!$B$6)</f>
@@ -5088,7 +5259,7 @@
         <v>0.85</v>
       </c>
       <c r="D26" s="0" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="E26" s="0" t="n">
         <f aca="false">(1-Supuestos!C$28)*((1+((1+Supuestos!C$26)/(1+Supuestos!$B$4)-1+Supuestos!$B$14*$A26/10000))*(1+Supuestos!$B$4+$B26/10000)-1)+Supuestos!C$28*((1+Supuestos!C$27+$A26/10000)*(1+Supuestos!$B$4+$B26/10000)-1)*(1-Supuestos!$B$6)</f>
@@ -5231,7 +5402,7 @@
         <v>0.85</v>
       </c>
       <c r="D27" s="0" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="E27" s="0" t="n">
         <f aca="false">(1-Supuestos!C$28)*((1+((1+Supuestos!C$26)/(1+Supuestos!$B$4)-1+Supuestos!$B$14*$A27/10000))*(1+Supuestos!$B$4+$B27/10000)-1)+Supuestos!C$28*((1+Supuestos!C$27+$A27/10000)*(1+Supuestos!$B$4+$B27/10000)-1)*(1-Supuestos!$B$6)</f>
@@ -5374,7 +5545,7 @@
         <v>0.85</v>
       </c>
       <c r="D28" s="0" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="E28" s="0" t="n">
         <f aca="false">(1-Supuestos!C$28)*((1+((1+Supuestos!C$26)/(1+Supuestos!$B$4)-1+Supuestos!$B$14*$A28/10000))*(1+Supuestos!$B$4+$B28/10000)-1)+Supuestos!C$28*((1+Supuestos!C$27+$A28/10000)*(1+Supuestos!$B$4+$B28/10000)-1)*(1-Supuestos!$B$6)</f>
@@ -5517,7 +5688,7 @@
         <v>0.85</v>
       </c>
       <c r="D29" s="0" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="E29" s="0" t="n">
         <f aca="false">(1-Supuestos!C$28)*((1+((1+Supuestos!C$26)/(1+Supuestos!$B$4)-1+Supuestos!$B$14*$A29/10000))*(1+Supuestos!$B$4+$B29/10000)-1)+Supuestos!C$28*((1+Supuestos!C$27+$A29/10000)*(1+Supuestos!$B$4+$B29/10000)-1)*(1-Supuestos!$B$6)</f>
@@ -5660,7 +5831,7 @@
         <v>0.85</v>
       </c>
       <c r="D30" s="0" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="E30" s="0" t="n">
         <f aca="false">(1-Supuestos!C$28)*((1+((1+Supuestos!C$26)/(1+Supuestos!$B$4)-1+Supuestos!$B$14*$A30/10000))*(1+Supuestos!$B$4+$B30/10000)-1)+Supuestos!C$28*((1+Supuestos!C$27+$A30/10000)*(1+Supuestos!$B$4+$B30/10000)-1)*(1-Supuestos!$B$6)</f>
@@ -5803,7 +5974,7 @@
         <v>0.85</v>
       </c>
       <c r="D31" s="0" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="E31" s="0" t="n">
         <f aca="false">(1-Supuestos!C$28)*((1+((1+Supuestos!C$26)/(1+Supuestos!$B$4)-1+Supuestos!$B$14*$A31/10000))*(1+Supuestos!$B$4+$B31/10000)-1)+Supuestos!C$28*((1+Supuestos!C$27+$A31/10000)*(1+Supuestos!$B$4+$B31/10000)-1)*(1-Supuestos!$B$6)</f>
@@ -5946,7 +6117,7 @@
         <v>0.85</v>
       </c>
       <c r="D32" s="0" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="E32" s="0" t="n">
         <f aca="false">(1-Supuestos!C$28)*((1+((1+Supuestos!C$26)/(1+Supuestos!$B$4)-1+Supuestos!$B$14*$A32/10000))*(1+Supuestos!$B$4+$B32/10000)-1)+Supuestos!C$28*((1+Supuestos!C$27+$A32/10000)*(1+Supuestos!$B$4+$B32/10000)-1)*(1-Supuestos!$B$6)</f>
@@ -6089,7 +6260,7 @@
         <v>0.85</v>
       </c>
       <c r="D33" s="0" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="E33" s="0" t="n">
         <f aca="false">(1-Supuestos!C$28)*((1+((1+Supuestos!C$26)/(1+Supuestos!$B$4)-1+Supuestos!$B$14*$A33/10000))*(1+Supuestos!$B$4+$B33/10000)-1)+Supuestos!C$28*((1+Supuestos!C$27+$A33/10000)*(1+Supuestos!$B$4+$B33/10000)-1)*(1-Supuestos!$B$6)</f>
@@ -6232,7 +6403,7 @@
         <v>0.85</v>
       </c>
       <c r="D34" s="0" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="E34" s="0" t="n">
         <f aca="false">(1-Supuestos!C$28)*((1+((1+Supuestos!C$26)/(1+Supuestos!$B$4)-1+Supuestos!$B$14*$A34/10000))*(1+Supuestos!$B$4+$B34/10000)-1)+Supuestos!C$28*((1+Supuestos!C$27+$A34/10000)*(1+Supuestos!$B$4+$B34/10000)-1)*(1-Supuestos!$B$6)</f>
@@ -6375,7 +6546,7 @@
         <v>0.85</v>
       </c>
       <c r="D35" s="0" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="E35" s="0" t="n">
         <f aca="false">(1-Supuestos!C$28)*((1+((1+Supuestos!C$26)/(1+Supuestos!$B$4)-1+Supuestos!$B$14*$A35/10000))*(1+Supuestos!$B$4+$B35/10000)-1)+Supuestos!C$28*((1+Supuestos!C$27+$A35/10000)*(1+Supuestos!$B$4+$B35/10000)-1)*(1-Supuestos!$B$6)</f>
@@ -6518,7 +6689,7 @@
         <v>0.85</v>
       </c>
       <c r="D36" s="0" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="E36" s="0" t="n">
         <f aca="false">(1-Supuestos!C$28)*((1+((1+Supuestos!C$26)/(1+Supuestos!$B$4)-1+Supuestos!$B$14*$A36/10000))*(1+Supuestos!$B$4+$B36/10000)-1)+Supuestos!C$28*((1+Supuestos!C$27+$A36/10000)*(1+Supuestos!$B$4+$B36/10000)-1)*(1-Supuestos!$B$6)</f>
@@ -6661,7 +6832,7 @@
         <v>0.85</v>
       </c>
       <c r="D37" s="0" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="E37" s="0" t="n">
         <f aca="false">(1-Supuestos!C$28)*((1+((1+Supuestos!C$26)/(1+Supuestos!$B$4)-1+Supuestos!$B$14*$A37/10000))*(1+Supuestos!$B$4+$B37/10000)-1)+Supuestos!C$28*((1+Supuestos!C$27+$A37/10000)*(1+Supuestos!$B$4+$B37/10000)-1)*(1-Supuestos!$B$6)</f>
@@ -6804,7 +6975,7 @@
         <v>0.85</v>
       </c>
       <c r="D38" s="0" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="E38" s="0" t="n">
         <f aca="false">(1-Supuestos!C$28)*((1+((1+Supuestos!C$26)/(1+Supuestos!$B$4)-1+Supuestos!$B$14*$A38/10000))*(1+Supuestos!$B$4+$B38/10000)-1)+Supuestos!C$28*((1+Supuestos!C$27+$A38/10000)*(1+Supuestos!$B$4+$B38/10000)-1)*(1-Supuestos!$B$6)</f>
@@ -6947,7 +7118,7 @@
         <v>0.85</v>
       </c>
       <c r="D39" s="0" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="E39" s="0" t="n">
         <f aca="false">(1-Supuestos!C$28)*((1+((1+Supuestos!C$26)/(1+Supuestos!$B$4)-1+Supuestos!$B$14*$A39/10000))*(1+Supuestos!$B$4+$B39/10000)-1)+Supuestos!C$28*((1+Supuestos!C$27+$A39/10000)*(1+Supuestos!$B$4+$B39/10000)-1)*(1-Supuestos!$B$6)</f>
@@ -7090,7 +7261,7 @@
         <v>0.85</v>
       </c>
       <c r="D40" s="0" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="E40" s="0" t="n">
         <f aca="false">(1-Supuestos!C$28)*((1+((1+Supuestos!C$26)/(1+Supuestos!$B$4)-1+Supuestos!$B$14*$A40/10000))*(1+Supuestos!$B$4+$B40/10000)-1)+Supuestos!C$28*((1+Supuestos!C$27+$A40/10000)*(1+Supuestos!$B$4+$B40/10000)-1)*(1-Supuestos!$B$6)</f>
@@ -7232,7 +7403,7 @@
         <v>1</v>
       </c>
       <c r="D41" s="0" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="E41" s="0" t="n">
         <f aca="false">(1-Supuestos!C$28)*((1+((1+Supuestos!C$26)/(1+Supuestos!$B$4)-1+Supuestos!$B$14*$A41/10000))*(1+Supuestos!$B$4+$B41/10000)-1)+Supuestos!C$28*((1+Supuestos!C$27+$A41/10000)*(1+Supuestos!$B$4+$B41/10000)-1)*(1-Supuestos!$B$6)</f>
@@ -7374,7 +7545,7 @@
         <v>1</v>
       </c>
       <c r="D42" s="0" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="E42" s="0" t="n">
         <f aca="false">(1-Supuestos!C$28)*((1+((1+Supuestos!C$26)/(1+Supuestos!$B$4)-1+Supuestos!$B$14*$A42/10000))*(1+Supuestos!$B$4+$B42/10000)-1)+Supuestos!C$28*((1+Supuestos!C$27+$A42/10000)*(1+Supuestos!$B$4+$B42/10000)-1)*(1-Supuestos!$B$6)</f>
@@ -7516,7 +7687,7 @@
         <v>1</v>
       </c>
       <c r="D43" s="0" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="E43" s="0" t="n">
         <f aca="false">(1-Supuestos!C$28)*((1+((1+Supuestos!C$26)/(1+Supuestos!$B$4)-1+Supuestos!$B$14*$A43/10000))*(1+Supuestos!$B$4+$B43/10000)-1)+Supuestos!C$28*((1+Supuestos!C$27+$A43/10000)*(1+Supuestos!$B$4+$B43/10000)-1)*(1-Supuestos!$B$6)</f>
@@ -7658,7 +7829,7 @@
         <v>1</v>
       </c>
       <c r="D44" s="0" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="E44" s="0" t="n">
         <f aca="false">(1-Supuestos!C$28)*((1+((1+Supuestos!C$26)/(1+Supuestos!$B$4)-1+Supuestos!$B$14*$A44/10000))*(1+Supuestos!$B$4+$B44/10000)-1)+Supuestos!C$28*((1+Supuestos!C$27+$A44/10000)*(1+Supuestos!$B$4+$B44/10000)-1)*(1-Supuestos!$B$6)</f>
@@ -7800,7 +7971,7 @@
         <v>1</v>
       </c>
       <c r="D45" s="0" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="E45" s="0" t="n">
         <f aca="false">(1-Supuestos!C$28)*((1+((1+Supuestos!C$26)/(1+Supuestos!$B$4)-1+Supuestos!$B$14*$A45/10000))*(1+Supuestos!$B$4+$B45/10000)-1)+Supuestos!C$28*((1+Supuestos!C$27+$A45/10000)*(1+Supuestos!$B$4+$B45/10000)-1)*(1-Supuestos!$B$6)</f>
@@ -7942,7 +8113,7 @@
         <v>1</v>
       </c>
       <c r="D46" s="0" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="E46" s="0" t="n">
         <f aca="false">(1-Supuestos!C$28)*((1+((1+Supuestos!C$26)/(1+Supuestos!$B$4)-1+Supuestos!$B$14*$A46/10000))*(1+Supuestos!$B$4+$B46/10000)-1)+Supuestos!C$28*((1+Supuestos!C$27+$A46/10000)*(1+Supuestos!$B$4+$B46/10000)-1)*(1-Supuestos!$B$6)</f>
@@ -8084,7 +8255,7 @@
         <v>1</v>
       </c>
       <c r="D47" s="0" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="E47" s="0" t="n">
         <f aca="false">(1-Supuestos!C$28)*((1+((1+Supuestos!C$26)/(1+Supuestos!$B$4)-1+Supuestos!$B$14*$A47/10000))*(1+Supuestos!$B$4+$B47/10000)-1)+Supuestos!C$28*((1+Supuestos!C$27+$A47/10000)*(1+Supuestos!$B$4+$B47/10000)-1)*(1-Supuestos!$B$6)</f>
@@ -8226,7 +8397,7 @@
         <v>1</v>
       </c>
       <c r="D48" s="0" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="E48" s="0" t="n">
         <f aca="false">(1-Supuestos!C$28)*((1+((1+Supuestos!C$26)/(1+Supuestos!$B$4)-1+Supuestos!$B$14*$A48/10000))*(1+Supuestos!$B$4+$B48/10000)-1)+Supuestos!C$28*((1+Supuestos!C$27+$A48/10000)*(1+Supuestos!$B$4+$B48/10000)-1)*(1-Supuestos!$B$6)</f>
@@ -8368,7 +8539,7 @@
         <v>1</v>
       </c>
       <c r="D49" s="0" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="E49" s="0" t="n">
         <f aca="false">(1-Supuestos!C$28)*((1+((1+Supuestos!C$26)/(1+Supuestos!$B$4)-1+Supuestos!$B$14*$A49/10000))*(1+Supuestos!$B$4+$B49/10000)-1)+Supuestos!C$28*((1+Supuestos!C$27+$A49/10000)*(1+Supuestos!$B$4+$B49/10000)-1)*(1-Supuestos!$B$6)</f>
@@ -8510,7 +8681,7 @@
         <v>1</v>
       </c>
       <c r="D50" s="0" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="E50" s="0" t="n">
         <f aca="false">(1-Supuestos!C$28)*((1+((1+Supuestos!C$26)/(1+Supuestos!$B$4)-1+Supuestos!$B$14*$A50/10000))*(1+Supuestos!$B$4+$B50/10000)-1)+Supuestos!C$28*((1+Supuestos!C$27+$A50/10000)*(1+Supuestos!$B$4+$B50/10000)-1)*(1-Supuestos!$B$6)</f>
@@ -8652,7 +8823,7 @@
         <v>1</v>
       </c>
       <c r="D51" s="0" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="E51" s="0" t="n">
         <f aca="false">(1-Supuestos!C$28)*((1+((1+Supuestos!C$26)/(1+Supuestos!$B$4)-1+Supuestos!$B$14*$A51/10000))*(1+Supuestos!$B$4+$B51/10000)-1)+Supuestos!C$28*((1+Supuestos!C$27+$A51/10000)*(1+Supuestos!$B$4+$B51/10000)-1)*(1-Supuestos!$B$6)</f>
@@ -8794,7 +8965,7 @@
         <v>0.85</v>
       </c>
       <c r="D52" s="0" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="E52" s="0" t="n">
         <f aca="false">(1-Supuestos!C$28)*((1+((1+Supuestos!C$26)/(1+Supuestos!$B$4)-1+Supuestos!$B$14*$A52/10000))*(1+Supuestos!$B$4+$B52/10000)-1)+Supuestos!C$28*((1+Supuestos!C$27+$A52/10000)*(1+Supuestos!$B$4+$B52/10000)-1)*(1-Supuestos!$B$6)</f>
@@ -8936,7 +9107,7 @@
         <v>0.85</v>
       </c>
       <c r="D53" s="0" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="E53" s="0" t="n">
         <f aca="false">(1-Supuestos!C$28)*((1+((1+Supuestos!C$26)/(1+Supuestos!$B$4)-1+Supuestos!$B$14*$A53/10000))*(1+Supuestos!$B$4+$B53/10000)-1)+Supuestos!C$28*((1+Supuestos!C$27+$A53/10000)*(1+Supuestos!$B$4+$B53/10000)-1)*(1-Supuestos!$B$6)</f>
@@ -9078,7 +9249,7 @@
         <v>0.85</v>
       </c>
       <c r="D54" s="0" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="E54" s="0" t="n">
         <f aca="false">(1-Supuestos!C$28)*((1+((1+Supuestos!C$26)/(1+Supuestos!$B$4)-1+Supuestos!$B$14*$A54/10000))*(1+Supuestos!$B$4+$B54/10000)-1)+Supuestos!C$28*((1+Supuestos!C$27+$A54/10000)*(1+Supuestos!$B$4+$B54/10000)-1)*(1-Supuestos!$B$6)</f>
@@ -9220,7 +9391,7 @@
         <v>0.85</v>
       </c>
       <c r="D55" s="0" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="E55" s="0" t="n">
         <f aca="false">(1-Supuestos!C$28)*((1+((1+Supuestos!C$26)/(1+Supuestos!$B$4)-1+Supuestos!$B$14*$A55/10000))*(1+Supuestos!$B$4+$B55/10000)-1)+Supuestos!C$28*((1+Supuestos!C$27+$A55/10000)*(1+Supuestos!$B$4+$B55/10000)-1)*(1-Supuestos!$B$6)</f>
@@ -9362,7 +9533,7 @@
         <v>0.85</v>
       </c>
       <c r="D56" s="0" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="E56" s="0" t="n">
         <f aca="false">(1-Supuestos!C$28)*((1+((1+Supuestos!C$26)/(1+Supuestos!$B$4)-1+Supuestos!$B$14*$A56/10000))*(1+Supuestos!$B$4+$B56/10000)-1)+Supuestos!C$28*((1+Supuestos!C$27+$A56/10000)*(1+Supuestos!$B$4+$B56/10000)-1)*(1-Supuestos!$B$6)</f>
@@ -9504,7 +9675,7 @@
         <v>0.85</v>
       </c>
       <c r="D57" s="0" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="E57" s="0" t="n">
         <f aca="false">(1-Supuestos!C$28)*((1+((1+Supuestos!C$26)/(1+Supuestos!$B$4)-1+Supuestos!$B$14*$A57/10000))*(1+Supuestos!$B$4+$B57/10000)-1)+Supuestos!C$28*((1+Supuestos!C$27+$A57/10000)*(1+Supuestos!$B$4+$B57/10000)-1)*(1-Supuestos!$B$6)</f>
@@ -9646,7 +9817,7 @@
         <v>0.85</v>
       </c>
       <c r="D58" s="0" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="E58" s="0" t="n">
         <f aca="false">(1-Supuestos!C$28)*((1+((1+Supuestos!C$26)/(1+Supuestos!$B$4)-1+Supuestos!$B$14*$A58/10000))*(1+Supuestos!$B$4+$B58/10000)-1)+Supuestos!C$28*((1+Supuestos!C$27+$A58/10000)*(1+Supuestos!$B$4+$B58/10000)-1)*(1-Supuestos!$B$6)</f>
@@ -9788,7 +9959,7 @@
         <v>0.85</v>
       </c>
       <c r="D59" s="0" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="E59" s="0" t="n">
         <f aca="false">(1-Supuestos!C$28)*((1+((1+Supuestos!C$26)/(1+Supuestos!$B$4)-1+Supuestos!$B$14*$A59/10000))*(1+Supuestos!$B$4+$B59/10000)-1)+Supuestos!C$28*((1+Supuestos!C$27+$A59/10000)*(1+Supuestos!$B$4+$B59/10000)-1)*(1-Supuestos!$B$6)</f>
@@ -9930,7 +10101,7 @@
         <v>0.85</v>
       </c>
       <c r="D60" s="0" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="E60" s="0" t="n">
         <f aca="false">(1-Supuestos!C$28)*((1+((1+Supuestos!C$26)/(1+Supuestos!$B$4)-1+Supuestos!$B$14*$A60/10000))*(1+Supuestos!$B$4+$B60/10000)-1)+Supuestos!C$28*((1+Supuestos!C$27+$A60/10000)*(1+Supuestos!$B$4+$B60/10000)-1)*(1-Supuestos!$B$6)</f>
@@ -10072,7 +10243,7 @@
         <v>0.85</v>
       </c>
       <c r="D61" s="0" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="E61" s="0" t="n">
         <f aca="false">(1-Supuestos!C$28)*((1+((1+Supuestos!C$26)/(1+Supuestos!$B$4)-1+Supuestos!$B$14*$A61/10000))*(1+Supuestos!$B$4+$B61/10000)-1)+Supuestos!C$28*((1+Supuestos!C$27+$A61/10000)*(1+Supuestos!$B$4+$B61/10000)-1)*(1-Supuestos!$B$6)</f>
@@ -10214,7 +10385,7 @@
         <v>0.85</v>
       </c>
       <c r="D62" s="0" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="E62" s="0" t="n">
         <f aca="false">(1-Supuestos!C$28)*((1+((1+Supuestos!C$26)/(1+Supuestos!$B$4)-1+Supuestos!$B$14*$A62/10000))*(1+Supuestos!$B$4+$B62/10000)-1)+Supuestos!C$28*((1+Supuestos!C$27+$A62/10000)*(1+Supuestos!$B$4+$B62/10000)-1)*(1-Supuestos!$B$6)</f>
@@ -10356,7 +10527,7 @@
         <v>0.7</v>
       </c>
       <c r="D63" s="0" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="E63" s="0" t="n">
         <f aca="false">(1-Supuestos!C$28)*((1+((1+Supuestos!C$26)/(1+Supuestos!$B$4)-1+Supuestos!$B$14*$A63/10000))*(1+Supuestos!$B$4+$B63/10000)-1)+Supuestos!C$28*((1+Supuestos!C$27+$A63/10000)*(1+Supuestos!$B$4+$B63/10000)-1)*(1-Supuestos!$B$6)</f>
@@ -10498,7 +10669,7 @@
         <v>0.7</v>
       </c>
       <c r="D64" s="0" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="E64" s="0" t="n">
         <f aca="false">(1-Supuestos!C$28)*((1+((1+Supuestos!C$26)/(1+Supuestos!$B$4)-1+Supuestos!$B$14*$A64/10000))*(1+Supuestos!$B$4+$B64/10000)-1)+Supuestos!C$28*((1+Supuestos!C$27+$A64/10000)*(1+Supuestos!$B$4+$B64/10000)-1)*(1-Supuestos!$B$6)</f>
@@ -10640,7 +10811,7 @@
         <v>0.7</v>
       </c>
       <c r="D65" s="0" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="E65" s="0" t="n">
         <f aca="false">(1-Supuestos!C$28)*((1+((1+Supuestos!C$26)/(1+Supuestos!$B$4)-1+Supuestos!$B$14*$A65/10000))*(1+Supuestos!$B$4+$B65/10000)-1)+Supuestos!C$28*((1+Supuestos!C$27+$A65/10000)*(1+Supuestos!$B$4+$B65/10000)-1)*(1-Supuestos!$B$6)</f>
@@ -10782,7 +10953,7 @@
         <v>0.7</v>
       </c>
       <c r="D66" s="0" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="E66" s="0" t="n">
         <f aca="false">(1-Supuestos!C$28)*((1+((1+Supuestos!C$26)/(1+Supuestos!$B$4)-1+Supuestos!$B$14*$A66/10000))*(1+Supuestos!$B$4+$B66/10000)-1)+Supuestos!C$28*((1+Supuestos!C$27+$A66/10000)*(1+Supuestos!$B$4+$B66/10000)-1)*(1-Supuestos!$B$6)</f>
@@ -10924,7 +11095,7 @@
         <v>0.7</v>
       </c>
       <c r="D67" s="0" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="E67" s="0" t="n">
         <f aca="false">(1-Supuestos!C$28)*((1+((1+Supuestos!C$26)/(1+Supuestos!$B$4)-1+Supuestos!$B$14*$A67/10000))*(1+Supuestos!$B$4+$B67/10000)-1)+Supuestos!C$28*((1+Supuestos!C$27+$A67/10000)*(1+Supuestos!$B$4+$B67/10000)-1)*(1-Supuestos!$B$6)</f>
@@ -11066,7 +11237,7 @@
         <v>0.7</v>
       </c>
       <c r="D68" s="0" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="E68" s="0" t="n">
         <f aca="false">(1-Supuestos!C$28)*((1+((1+Supuestos!C$26)/(1+Supuestos!$B$4)-1+Supuestos!$B$14*$A68/10000))*(1+Supuestos!$B$4+$B68/10000)-1)+Supuestos!C$28*((1+Supuestos!C$27+$A68/10000)*(1+Supuestos!$B$4+$B68/10000)-1)*(1-Supuestos!$B$6)</f>
@@ -11208,7 +11379,7 @@
         <v>0.7</v>
       </c>
       <c r="D69" s="0" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="E69" s="0" t="n">
         <f aca="false">(1-Supuestos!C$28)*((1+((1+Supuestos!C$26)/(1+Supuestos!$B$4)-1+Supuestos!$B$14*$A69/10000))*(1+Supuestos!$B$4+$B69/10000)-1)+Supuestos!C$28*((1+Supuestos!C$27+$A69/10000)*(1+Supuestos!$B$4+$B69/10000)-1)*(1-Supuestos!$B$6)</f>
@@ -11350,7 +11521,7 @@
         <v>0.7</v>
       </c>
       <c r="D70" s="0" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="E70" s="0" t="n">
         <f aca="false">(1-Supuestos!C$28)*((1+((1+Supuestos!C$26)/(1+Supuestos!$B$4)-1+Supuestos!$B$14*$A70/10000))*(1+Supuestos!$B$4+$B70/10000)-1)+Supuestos!C$28*((1+Supuestos!C$27+$A70/10000)*(1+Supuestos!$B$4+$B70/10000)-1)*(1-Supuestos!$B$6)</f>
@@ -11492,7 +11663,7 @@
         <v>0.7</v>
       </c>
       <c r="D71" s="0" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="E71" s="0" t="n">
         <f aca="false">(1-Supuestos!C$28)*((1+((1+Supuestos!C$26)/(1+Supuestos!$B$4)-1+Supuestos!$B$14*$A71/10000))*(1+Supuestos!$B$4+$B71/10000)-1)+Supuestos!C$28*((1+Supuestos!C$27+$A71/10000)*(1+Supuestos!$B$4+$B71/10000)-1)*(1-Supuestos!$B$6)</f>
@@ -11634,7 +11805,7 @@
         <v>0.7</v>
       </c>
       <c r="D72" s="0" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="E72" s="0" t="n">
         <f aca="false">(1-Supuestos!C$28)*((1+((1+Supuestos!C$26)/(1+Supuestos!$B$4)-1+Supuestos!$B$14*$A72/10000))*(1+Supuestos!$B$4+$B72/10000)-1)+Supuestos!C$28*((1+Supuestos!C$27+$A72/10000)*(1+Supuestos!$B$4+$B72/10000)-1)*(1-Supuestos!$B$6)</f>
@@ -11776,7 +11947,7 @@
         <v>0.7</v>
       </c>
       <c r="D73" s="0" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="E73" s="0" t="n">
         <f aca="false">(1-Supuestos!C$28)*((1+((1+Supuestos!C$26)/(1+Supuestos!$B$4)-1+Supuestos!$B$14*$A73/10000))*(1+Supuestos!$B$4+$B73/10000)-1)+Supuestos!C$28*((1+Supuestos!C$27+$A73/10000)*(1+Supuestos!$B$4+$B73/10000)-1)*(1-Supuestos!$B$6)</f>
@@ -11918,7 +12089,7 @@
         <v>1</v>
       </c>
       <c r="D74" s="0" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
       <c r="E74" s="0" t="n">
         <f aca="false">(1-Supuestos!C$28)*((1+((1+Supuestos!C$26)/(1+Supuestos!$B$4)-1+Supuestos!$B$14*$A74/10000))*(1+Supuestos!$B$4+$B74/10000)-1)+Supuestos!C$28*((1+Supuestos!C$27+$A74/10000)*(1+Supuestos!$B$4+$B74/10000)-1)*(1-Supuestos!$B$6)</f>
@@ -12060,7 +12231,7 @@
         <v>1</v>
       </c>
       <c r="D75" s="0" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
       <c r="E75" s="0" t="n">
         <f aca="false">(1-Supuestos!C$28)*((1+((1+Supuestos!C$26)/(1+Supuestos!$B$4)-1+Supuestos!$B$14*$A75/10000))*(1+Supuestos!$B$4+$B75/10000)-1)+Supuestos!C$28*((1+Supuestos!C$27+$A75/10000)*(1+Supuestos!$B$4+$B75/10000)-1)*(1-Supuestos!$B$6)</f>
@@ -12202,7 +12373,7 @@
         <v>1</v>
       </c>
       <c r="D76" s="0" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
       <c r="E76" s="0" t="n">
         <f aca="false">(1-Supuestos!C$28)*((1+((1+Supuestos!C$26)/(1+Supuestos!$B$4)-1+Supuestos!$B$14*$A76/10000))*(1+Supuestos!$B$4+$B76/10000)-1)+Supuestos!C$28*((1+Supuestos!C$27+$A76/10000)*(1+Supuestos!$B$4+$B76/10000)-1)*(1-Supuestos!$B$6)</f>
@@ -12344,7 +12515,7 @@
         <v>1</v>
       </c>
       <c r="D77" s="0" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
       <c r="E77" s="0" t="n">
         <f aca="false">(1-Supuestos!C$28)*((1+((1+Supuestos!C$26)/(1+Supuestos!$B$4)-1+Supuestos!$B$14*$A77/10000))*(1+Supuestos!$B$4+$B77/10000)-1)+Supuestos!C$28*((1+Supuestos!C$27+$A77/10000)*(1+Supuestos!$B$4+$B77/10000)-1)*(1-Supuestos!$B$6)</f>
@@ -12486,7 +12657,7 @@
         <v>1</v>
       </c>
       <c r="D78" s="0" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
       <c r="E78" s="0" t="n">
         <f aca="false">(1-Supuestos!C$28)*((1+((1+Supuestos!C$26)/(1+Supuestos!$B$4)-1+Supuestos!$B$14*$A78/10000))*(1+Supuestos!$B$4+$B78/10000)-1)+Supuestos!C$28*((1+Supuestos!C$27+$A78/10000)*(1+Supuestos!$B$4+$B78/10000)-1)*(1-Supuestos!$B$6)</f>
@@ -12628,7 +12799,7 @@
         <v>1</v>
       </c>
       <c r="D79" s="0" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
       <c r="E79" s="0" t="n">
         <f aca="false">(1-Supuestos!C$28)*((1+((1+Supuestos!C$26)/(1+Supuestos!$B$4)-1+Supuestos!$B$14*$A79/10000))*(1+Supuestos!$B$4+$B79/10000)-1)+Supuestos!C$28*((1+Supuestos!C$27+$A79/10000)*(1+Supuestos!$B$4+$B79/10000)-1)*(1-Supuestos!$B$6)</f>
@@ -12770,7 +12941,7 @@
         <v>1</v>
       </c>
       <c r="D80" s="0" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
       <c r="E80" s="0" t="n">
         <f aca="false">(1-Supuestos!C$28)*((1+((1+Supuestos!C$26)/(1+Supuestos!$B$4)-1+Supuestos!$B$14*$A80/10000))*(1+Supuestos!$B$4+$B80/10000)-1)+Supuestos!C$28*((1+Supuestos!C$27+$A80/10000)*(1+Supuestos!$B$4+$B80/10000)-1)*(1-Supuestos!$B$6)</f>
@@ -12912,7 +13083,7 @@
         <v>1</v>
       </c>
       <c r="D81" s="0" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
       <c r="E81" s="0" t="n">
         <f aca="false">(1-Supuestos!C$28)*((1+((1+Supuestos!C$26)/(1+Supuestos!$B$4)-1+Supuestos!$B$14*$A81/10000))*(1+Supuestos!$B$4+$B81/10000)-1)+Supuestos!C$28*((1+Supuestos!C$27+$A81/10000)*(1+Supuestos!$B$4+$B81/10000)-1)*(1-Supuestos!$B$6)</f>
@@ -13054,7 +13225,7 @@
         <v>1</v>
       </c>
       <c r="D82" s="0" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
       <c r="E82" s="0" t="n">
         <f aca="false">(1-Supuestos!C$28)*((1+((1+Supuestos!C$26)/(1+Supuestos!$B$4)-1+Supuestos!$B$14*$A82/10000))*(1+Supuestos!$B$4+$B82/10000)-1)+Supuestos!C$28*((1+Supuestos!C$27+$A82/10000)*(1+Supuestos!$B$4+$B82/10000)-1)*(1-Supuestos!$B$6)</f>
@@ -13196,7 +13367,7 @@
         <v>1</v>
       </c>
       <c r="D83" s="0" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
       <c r="E83" s="0" t="n">
         <f aca="false">(1-Supuestos!C$28)*((1+((1+Supuestos!C$26)/(1+Supuestos!$B$4)-1+Supuestos!$B$14*$A83/10000))*(1+Supuestos!$B$4+$B83/10000)-1)+Supuestos!C$28*((1+Supuestos!C$27+$A83/10000)*(1+Supuestos!$B$4+$B83/10000)-1)*(1-Supuestos!$B$6)</f>
@@ -13338,7 +13509,7 @@
         <v>1</v>
       </c>
       <c r="D84" s="0" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
       <c r="E84" s="0" t="n">
         <f aca="false">(1-Supuestos!C$28)*((1+((1+Supuestos!C$26)/(1+Supuestos!$B$4)-1+Supuestos!$B$14*$A84/10000))*(1+Supuestos!$B$4+$B84/10000)-1)+Supuestos!C$28*((1+Supuestos!C$27+$A84/10000)*(1+Supuestos!$B$4+$B84/10000)-1)*(1-Supuestos!$B$6)</f>
@@ -13480,7 +13651,7 @@
         <v>0.85</v>
       </c>
       <c r="D85" s="0" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="E85" s="0" t="n">
         <f aca="false">(1-Supuestos!C$28)*((1+((1+Supuestos!C$26)/(1+Supuestos!$B$4)-1+Supuestos!$B$14*$A85/10000))*(1+Supuestos!$B$4+$B85/10000)-1)+Supuestos!C$28*((1+Supuestos!C$27+$A85/10000)*(1+Supuestos!$B$4+$B85/10000)-1)*(1-Supuestos!$B$6)</f>
@@ -13622,7 +13793,7 @@
         <v>0.85</v>
       </c>
       <c r="D86" s="0" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="E86" s="0" t="n">
         <f aca="false">(1-Supuestos!C$28)*((1+((1+Supuestos!C$26)/(1+Supuestos!$B$4)-1+Supuestos!$B$14*$A86/10000))*(1+Supuestos!$B$4+$B86/10000)-1)+Supuestos!C$28*((1+Supuestos!C$27+$A86/10000)*(1+Supuestos!$B$4+$B86/10000)-1)*(1-Supuestos!$B$6)</f>
@@ -13764,7 +13935,7 @@
         <v>0.85</v>
       </c>
       <c r="D87" s="0" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="E87" s="0" t="n">
         <f aca="false">(1-Supuestos!C$28)*((1+((1+Supuestos!C$26)/(1+Supuestos!$B$4)-1+Supuestos!$B$14*$A87/10000))*(1+Supuestos!$B$4+$B87/10000)-1)+Supuestos!C$28*((1+Supuestos!C$27+$A87/10000)*(1+Supuestos!$B$4+$B87/10000)-1)*(1-Supuestos!$B$6)</f>
@@ -13906,7 +14077,7 @@
         <v>0.85</v>
       </c>
       <c r="D88" s="0" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="E88" s="0" t="n">
         <f aca="false">(1-Supuestos!C$28)*((1+((1+Supuestos!C$26)/(1+Supuestos!$B$4)-1+Supuestos!$B$14*$A88/10000))*(1+Supuestos!$B$4+$B88/10000)-1)+Supuestos!C$28*((1+Supuestos!C$27+$A88/10000)*(1+Supuestos!$B$4+$B88/10000)-1)*(1-Supuestos!$B$6)</f>
@@ -14048,7 +14219,7 @@
         <v>0.85</v>
       </c>
       <c r="D89" s="0" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="E89" s="0" t="n">
         <f aca="false">(1-Supuestos!C$28)*((1+((1+Supuestos!C$26)/(1+Supuestos!$B$4)-1+Supuestos!$B$14*$A89/10000))*(1+Supuestos!$B$4+$B89/10000)-1)+Supuestos!C$28*((1+Supuestos!C$27+$A89/10000)*(1+Supuestos!$B$4+$B89/10000)-1)*(1-Supuestos!$B$6)</f>
@@ -14190,7 +14361,7 @@
         <v>0.85</v>
       </c>
       <c r="D90" s="0" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="E90" s="0" t="n">
         <f aca="false">(1-Supuestos!C$28)*((1+((1+Supuestos!C$26)/(1+Supuestos!$B$4)-1+Supuestos!$B$14*$A90/10000))*(1+Supuestos!$B$4+$B90/10000)-1)+Supuestos!C$28*((1+Supuestos!C$27+$A90/10000)*(1+Supuestos!$B$4+$B90/10000)-1)*(1-Supuestos!$B$6)</f>
@@ -14332,7 +14503,7 @@
         <v>0.85</v>
       </c>
       <c r="D91" s="0" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="E91" s="0" t="n">
         <f aca="false">(1-Supuestos!C$28)*((1+((1+Supuestos!C$26)/(1+Supuestos!$B$4)-1+Supuestos!$B$14*$A91/10000))*(1+Supuestos!$B$4+$B91/10000)-1)+Supuestos!C$28*((1+Supuestos!C$27+$A91/10000)*(1+Supuestos!$B$4+$B91/10000)-1)*(1-Supuestos!$B$6)</f>
@@ -14474,7 +14645,7 @@
         <v>0.85</v>
       </c>
       <c r="D92" s="0" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="E92" s="0" t="n">
         <f aca="false">(1-Supuestos!C$28)*((1+((1+Supuestos!C$26)/(1+Supuestos!$B$4)-1+Supuestos!$B$14*$A92/10000))*(1+Supuestos!$B$4+$B92/10000)-1)+Supuestos!C$28*((1+Supuestos!C$27+$A92/10000)*(1+Supuestos!$B$4+$B92/10000)-1)*(1-Supuestos!$B$6)</f>
@@ -14616,7 +14787,7 @@
         <v>0.85</v>
       </c>
       <c r="D93" s="0" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="E93" s="0" t="n">
         <f aca="false">(1-Supuestos!C$28)*((1+((1+Supuestos!C$26)/(1+Supuestos!$B$4)-1+Supuestos!$B$14*$A93/10000))*(1+Supuestos!$B$4+$B93/10000)-1)+Supuestos!C$28*((1+Supuestos!C$27+$A93/10000)*(1+Supuestos!$B$4+$B93/10000)-1)*(1-Supuestos!$B$6)</f>
@@ -14758,7 +14929,7 @@
         <v>0.85</v>
       </c>
       <c r="D94" s="0" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="E94" s="0" t="n">
         <f aca="false">(1-Supuestos!C$28)*((1+((1+Supuestos!C$26)/(1+Supuestos!$B$4)-1+Supuestos!$B$14*$A94/10000))*(1+Supuestos!$B$4+$B94/10000)-1)+Supuestos!C$28*((1+Supuestos!C$27+$A94/10000)*(1+Supuestos!$B$4+$B94/10000)-1)*(1-Supuestos!$B$6)</f>
@@ -14900,7 +15071,7 @@
         <v>0.85</v>
       </c>
       <c r="D95" s="0" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="E95" s="0" t="n">
         <f aca="false">(1-Supuestos!C$28)*((1+((1+Supuestos!C$26)/(1+Supuestos!$B$4)-1+Supuestos!$B$14*$A95/10000))*(1+Supuestos!$B$4+$B95/10000)-1)+Supuestos!C$28*((1+Supuestos!C$27+$A95/10000)*(1+Supuestos!$B$4+$B95/10000)-1)*(1-Supuestos!$B$6)</f>
@@ -15042,7 +15213,7 @@
         <v>0.7</v>
       </c>
       <c r="D96" s="0" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="E96" s="0" t="n">
         <f aca="false">(1-Supuestos!C$28)*((1+((1+Supuestos!C$26)/(1+Supuestos!$B$4)-1+Supuestos!$B$14*$A96/10000))*(1+Supuestos!$B$4+$B96/10000)-1)+Supuestos!C$28*((1+Supuestos!C$27+$A96/10000)*(1+Supuestos!$B$4+$B96/10000)-1)*(1-Supuestos!$B$6)</f>
@@ -15184,7 +15355,7 @@
         <v>0.7</v>
       </c>
       <c r="D97" s="0" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="E97" s="0" t="n">
         <f aca="false">(1-Supuestos!C$28)*((1+((1+Supuestos!C$26)/(1+Supuestos!$B$4)-1+Supuestos!$B$14*$A97/10000))*(1+Supuestos!$B$4+$B97/10000)-1)+Supuestos!C$28*((1+Supuestos!C$27+$A97/10000)*(1+Supuestos!$B$4+$B97/10000)-1)*(1-Supuestos!$B$6)</f>
@@ -15326,7 +15497,7 @@
         <v>0.7</v>
       </c>
       <c r="D98" s="0" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="E98" s="0" t="n">
         <f aca="false">(1-Supuestos!C$28)*((1+((1+Supuestos!C$26)/(1+Supuestos!$B$4)-1+Supuestos!$B$14*$A98/10000))*(1+Supuestos!$B$4+$B98/10000)-1)+Supuestos!C$28*((1+Supuestos!C$27+$A98/10000)*(1+Supuestos!$B$4+$B98/10000)-1)*(1-Supuestos!$B$6)</f>
@@ -15468,7 +15639,7 @@
         <v>0.7</v>
       </c>
       <c r="D99" s="0" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="E99" s="0" t="n">
         <f aca="false">(1-Supuestos!C$28)*((1+((1+Supuestos!C$26)/(1+Supuestos!$B$4)-1+Supuestos!$B$14*$A99/10000))*(1+Supuestos!$B$4+$B99/10000)-1)+Supuestos!C$28*((1+Supuestos!C$27+$A99/10000)*(1+Supuestos!$B$4+$B99/10000)-1)*(1-Supuestos!$B$6)</f>
@@ -15610,7 +15781,7 @@
         <v>0.7</v>
       </c>
       <c r="D100" s="0" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="E100" s="0" t="n">
         <f aca="false">(1-Supuestos!C$28)*((1+((1+Supuestos!C$26)/(1+Supuestos!$B$4)-1+Supuestos!$B$14*$A100/10000))*(1+Supuestos!$B$4+$B100/10000)-1)+Supuestos!C$28*((1+Supuestos!C$27+$A100/10000)*(1+Supuestos!$B$4+$B100/10000)-1)*(1-Supuestos!$B$6)</f>
@@ -15752,7 +15923,7 @@
         <v>0.7</v>
       </c>
       <c r="D101" s="0" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="E101" s="0" t="n">
         <f aca="false">(1-Supuestos!C$28)*((1+((1+Supuestos!C$26)/(1+Supuestos!$B$4)-1+Supuestos!$B$14*$A101/10000))*(1+Supuestos!$B$4+$B101/10000)-1)+Supuestos!C$28*((1+Supuestos!C$27+$A101/10000)*(1+Supuestos!$B$4+$B101/10000)-1)*(1-Supuestos!$B$6)</f>
@@ -15894,7 +16065,7 @@
         <v>0.7</v>
       </c>
       <c r="D102" s="0" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="E102" s="0" t="n">
         <f aca="false">(1-Supuestos!C$28)*((1+((1+Supuestos!C$26)/(1+Supuestos!$B$4)-1+Supuestos!$B$14*$A102/10000))*(1+Supuestos!$B$4+$B102/10000)-1)+Supuestos!C$28*((1+Supuestos!C$27+$A102/10000)*(1+Supuestos!$B$4+$B102/10000)-1)*(1-Supuestos!$B$6)</f>
@@ -16036,7 +16207,7 @@
         <v>0.7</v>
       </c>
       <c r="D103" s="0" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="E103" s="0" t="n">
         <f aca="false">(1-Supuestos!C$28)*((1+((1+Supuestos!C$26)/(1+Supuestos!$B$4)-1+Supuestos!$B$14*$A103/10000))*(1+Supuestos!$B$4+$B103/10000)-1)+Supuestos!C$28*((1+Supuestos!C$27+$A103/10000)*(1+Supuestos!$B$4+$B103/10000)-1)*(1-Supuestos!$B$6)</f>
@@ -16178,7 +16349,7 @@
         <v>0.7</v>
       </c>
       <c r="D104" s="0" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="E104" s="0" t="n">
         <f aca="false">(1-Supuestos!C$28)*((1+((1+Supuestos!C$26)/(1+Supuestos!$B$4)-1+Supuestos!$B$14*$A104/10000))*(1+Supuestos!$B$4+$B104/10000)-1)+Supuestos!C$28*((1+Supuestos!C$27+$A104/10000)*(1+Supuestos!$B$4+$B104/10000)-1)*(1-Supuestos!$B$6)</f>
@@ -16320,7 +16491,7 @@
         <v>0.7</v>
       </c>
       <c r="D105" s="0" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="E105" s="0" t="n">
         <f aca="false">(1-Supuestos!C$28)*((1+((1+Supuestos!C$26)/(1+Supuestos!$B$4)-1+Supuestos!$B$14*$A105/10000))*(1+Supuestos!$B$4+$B105/10000)-1)+Supuestos!C$28*((1+Supuestos!C$27+$A105/10000)*(1+Supuestos!$B$4+$B105/10000)-1)*(1-Supuestos!$B$6)</f>
@@ -16462,7 +16633,7 @@
         <v>0.7</v>
       </c>
       <c r="D106" s="0" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="E106" s="0" t="n">
         <f aca="false">(1-Supuestos!C$28)*((1+((1+Supuestos!C$26)/(1+Supuestos!$B$4)-1+Supuestos!$B$14*$A106/10000))*(1+Supuestos!$B$4+$B106/10000)-1)+Supuestos!C$28*((1+Supuestos!C$27+$A106/10000)*(1+Supuestos!$B$4+$B106/10000)-1)*(1-Supuestos!$B$6)</f>
@@ -16607,7 +16778,7 @@
         <v>0.85</v>
       </c>
       <c r="D107" s="0" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="E107" s="0" t="n">
         <f aca="false">(1-Supuestos!C$28)*((1+((1+Supuestos!C$26)/(1+Supuestos!$B$4)-1+Supuestos!$B$14*$A107/10000))*(1+Supuestos!$B$4+$B107/10000)-1)+Supuestos!C$28*((1+Supuestos!C$27+$A107/10000)*(1+Supuestos!$B$4+$B107/10000)-1)*(1-Supuestos!$B$6)</f>
@@ -16759,60 +16930,60 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="0" t="s">
-        <v>119</v>
+        <v>121</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="0" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="0" t="s">
-        <v>121</v>
+        <v>123</v>
       </c>
       <c r="B4" s="0" t="s">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="C4" s="0" t="s">
-        <v>123</v>
+        <v>125</v>
       </c>
       <c r="D4" s="0" t="s">
-        <v>124</v>
+        <v>126</v>
       </c>
       <c r="E4" s="0" t="s">
-        <v>125</v>
+        <v>127</v>
       </c>
       <c r="F4" s="0" t="s">
-        <v>126</v>
+        <v>128</v>
       </c>
       <c r="G4" s="0" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
       <c r="H4" s="0" t="s">
-        <v>128</v>
+        <v>130</v>
       </c>
       <c r="I4" s="0" t="s">
-        <v>129</v>
+        <v>131</v>
       </c>
       <c r="J4" s="0" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="6" t="n">
+      <c r="A5" s="7" t="n">
         <v>45478</v>
       </c>
-      <c r="B5" s="3" t="n">
+      <c r="B5" s="5" t="n">
         <v>1381.56</v>
       </c>
-      <c r="C5" s="3" t="n">
+      <c r="C5" s="5" t="n">
         <v>6.22</v>
       </c>
-      <c r="D5" s="3" t="n">
+      <c r="D5" s="5" t="n">
         <v>3.1</v>
       </c>
-      <c r="E5" s="3" t="n">
+      <c r="E5" s="5" t="n">
         <v>6483.67</v>
       </c>
       <c r="F5" s="4" t="n">
@@ -16821,19 +16992,19 @@
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="6" t="n">
+      <c r="A6" s="7" t="n">
         <v>45485</v>
       </c>
-      <c r="B6" s="3" t="n">
+      <c r="B6" s="5" t="n">
         <v>1362.81</v>
       </c>
-      <c r="C6" s="3" t="n">
+      <c r="C6" s="5" t="n">
         <v>6.11</v>
       </c>
-      <c r="D6" s="3" t="n">
+      <c r="D6" s="5" t="n">
         <v>2.9</v>
       </c>
-      <c r="E6" s="3" t="n">
+      <c r="E6" s="5" t="n">
         <v>6550.01</v>
       </c>
       <c r="F6" s="4" t="n">
@@ -16858,19 +17029,19 @@
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="6" t="n">
+      <c r="A7" s="7" t="n">
         <v>45492</v>
       </c>
-      <c r="B7" s="3" t="n">
+      <c r="B7" s="5" t="n">
         <v>1421.03</v>
       </c>
-      <c r="C7" s="3" t="n">
+      <c r="C7" s="5" t="n">
         <v>6.1</v>
       </c>
-      <c r="D7" s="3" t="n">
+      <c r="D7" s="5" t="n">
         <v>2.87</v>
       </c>
-      <c r="E7" s="3" t="n">
+      <c r="E7" s="5" t="n">
         <v>6558.68</v>
       </c>
       <c r="F7" s="4" t="n">
@@ -16895,19 +17066,19 @@
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="6" t="n">
+      <c r="A8" s="7" t="n">
         <v>45499</v>
       </c>
-      <c r="B8" s="3" t="n">
+      <c r="B8" s="5" t="n">
         <v>1440.77</v>
       </c>
-      <c r="C8" s="3" t="n">
+      <c r="C8" s="5" t="n">
         <v>6.08</v>
       </c>
-      <c r="D8" s="3" t="n">
+      <c r="D8" s="5" t="n">
         <v>2.77</v>
       </c>
-      <c r="E8" s="3" t="n">
+      <c r="E8" s="5" t="n">
         <v>6432.16</v>
       </c>
       <c r="F8" s="4" t="n">
@@ -16932,19 +17103,19 @@
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="6" t="n">
+      <c r="A9" s="7" t="n">
         <v>45506</v>
       </c>
-      <c r="B9" s="3" t="n">
+      <c r="B9" s="5" t="n">
         <v>1423.4</v>
       </c>
-      <c r="C9" s="3" t="n">
+      <c r="C9" s="5" t="n">
         <v>5.99</v>
       </c>
-      <c r="D9" s="3" t="n">
+      <c r="D9" s="5" t="n">
         <v>2.6</v>
       </c>
-      <c r="E9" s="3" t="n">
+      <c r="E9" s="5" t="n">
         <v>6315.46</v>
       </c>
       <c r="F9" s="4" t="n">
@@ -16969,19 +17140,19 @@
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="6" t="n">
+      <c r="A10" s="7" t="n">
         <v>45513</v>
       </c>
-      <c r="B10" s="3" t="n">
+      <c r="B10" s="5" t="n">
         <v>1460.5</v>
       </c>
-      <c r="C10" s="3" t="n">
+      <c r="C10" s="5" t="n">
         <v>5.91</v>
       </c>
-      <c r="D10" s="3" t="n">
+      <c r="D10" s="5" t="n">
         <v>2.53</v>
       </c>
-      <c r="E10" s="3" t="n">
+      <c r="E10" s="5" t="n">
         <v>6320.96</v>
       </c>
       <c r="F10" s="4" t="n">
@@ -17006,19 +17177,19 @@
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="6" t="n">
+      <c r="A11" s="7" t="n">
         <v>45520</v>
       </c>
-      <c r="B11" s="3" t="n">
+      <c r="B11" s="5" t="n">
         <v>1512.11</v>
       </c>
-      <c r="C11" s="3" t="n">
+      <c r="C11" s="5" t="n">
         <v>5.8</v>
       </c>
-      <c r="D11" s="3" t="n">
+      <c r="D11" s="5" t="n">
         <v>2.49</v>
       </c>
-      <c r="E11" s="3" t="n">
+      <c r="E11" s="5" t="n">
         <v>6457.74</v>
       </c>
       <c r="F11" s="4" t="n">
@@ -17043,19 +17214,19 @@
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="6" t="n">
+      <c r="A12" s="7" t="n">
         <v>45527</v>
       </c>
-      <c r="B12" s="3" t="n">
+      <c r="B12" s="5" t="n">
         <v>1519.71</v>
       </c>
-      <c r="C12" s="3" t="n">
+      <c r="C12" s="5" t="n">
         <v>5.73</v>
       </c>
-      <c r="D12" s="3" t="n">
+      <c r="D12" s="5" t="n">
         <v>2.4</v>
       </c>
-      <c r="E12" s="3" t="n">
+      <c r="E12" s="5" t="n">
         <v>6463.24</v>
       </c>
       <c r="F12" s="4" t="n">
@@ -17080,19 +17251,19 @@
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="6" t="n">
+      <c r="A13" s="7" t="n">
         <v>45534</v>
       </c>
-      <c r="B13" s="3" t="n">
+      <c r="B13" s="5" t="n">
         <v>1490.21</v>
       </c>
-      <c r="C13" s="3" t="n">
+      <c r="C13" s="5" t="n">
         <v>5.64</v>
       </c>
-      <c r="D13" s="3" t="n">
+      <c r="D13" s="5" t="n">
         <v>2.37</v>
       </c>
-      <c r="E13" s="3" t="n">
+      <c r="E13" s="5" t="n">
         <v>6459.96</v>
       </c>
       <c r="F13" s="4" t="n">
@@ -17117,19 +17288,19 @@
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="6" t="n">
+      <c r="A14" s="7" t="n">
         <v>45541</v>
       </c>
-      <c r="B14" s="3" t="n">
+      <c r="B14" s="5" t="n">
         <v>1506.29</v>
       </c>
-      <c r="C14" s="3" t="n">
+      <c r="C14" s="5" t="n">
         <v>5.5</v>
       </c>
-      <c r="D14" s="3" t="n">
+      <c r="D14" s="5" t="n">
         <v>2.26</v>
       </c>
-      <c r="E14" s="3" t="n">
+      <c r="E14" s="5" t="n">
         <v>6245.42</v>
       </c>
       <c r="F14" s="4" t="n">
@@ -17154,19 +17325,19 @@
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="6" t="n">
+      <c r="A15" s="7" t="n">
         <v>45547</v>
       </c>
-      <c r="B15" s="3" t="n">
+      <c r="B15" s="5" t="n">
         <v>1509.05</v>
       </c>
-      <c r="C15" s="3" t="n">
+      <c r="C15" s="5" t="n">
         <v>5.37</v>
       </c>
-      <c r="D15" s="3" t="n">
+      <c r="D15" s="5" t="n">
         <v>2.1</v>
       </c>
-      <c r="E15" s="3" t="n">
+      <c r="E15" s="5" t="n">
         <v>6343.16</v>
       </c>
       <c r="F15" s="4" t="n">
@@ -17191,19 +17362,19 @@
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="6" t="n">
+      <c r="A16" s="7" t="n">
         <v>45562</v>
       </c>
-      <c r="B16" s="3" t="n">
+      <c r="B16" s="5" t="n">
         <v>1580.6</v>
       </c>
-      <c r="C16" s="3" t="n">
+      <c r="C16" s="5" t="n">
         <v>5.16</v>
       </c>
-      <c r="D16" s="3" t="n">
+      <c r="D16" s="5" t="n">
         <v>1.82</v>
       </c>
-      <c r="E16" s="3" t="n">
+      <c r="E16" s="5" t="n">
         <v>6530.73</v>
       </c>
       <c r="F16" s="4" t="n">
@@ -17228,19 +17399,19 @@
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="6" t="n">
+      <c r="A17" s="7" t="n">
         <v>45568</v>
       </c>
-      <c r="B17" s="3" t="n">
+      <c r="B17" s="5" t="n">
         <v>1524.65</v>
       </c>
-      <c r="C17" s="3" t="n">
+      <c r="C17" s="5" t="n">
         <v>5.3</v>
       </c>
-      <c r="D17" s="3" t="n">
+      <c r="D17" s="5" t="n">
         <v>2</v>
       </c>
-      <c r="E17" s="3" t="n">
+      <c r="E17" s="5" t="n">
         <v>6389.82</v>
       </c>
       <c r="F17" s="4" t="n">
@@ -17265,19 +17436,19 @@
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="6" t="n">
+      <c r="A18" s="7" t="n">
         <v>45575</v>
       </c>
-      <c r="B18" s="3" t="n">
+      <c r="B18" s="5" t="n">
         <v>1588.79</v>
       </c>
-      <c r="C18" s="3" t="n">
+      <c r="C18" s="5" t="n">
         <v>5.57</v>
       </c>
-      <c r="D18" s="3" t="n">
+      <c r="D18" s="5" t="n">
         <v>2.31</v>
       </c>
-      <c r="E18" s="3" t="n">
+      <c r="E18" s="5" t="n">
         <v>6578.77</v>
       </c>
       <c r="F18" s="4" t="n">
@@ -17302,19 +17473,19 @@
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="6" t="n">
+      <c r="A19" s="7" t="n">
         <v>45583</v>
       </c>
-      <c r="B19" s="3" t="n">
+      <c r="B19" s="5" t="n">
         <v>1569.05</v>
       </c>
-      <c r="C19" s="3" t="n">
+      <c r="C19" s="5" t="n">
         <v>5.49</v>
       </c>
-      <c r="D19" s="3" t="n">
+      <c r="D19" s="5" t="n">
         <v>2.21</v>
       </c>
-      <c r="E19" s="3" t="n">
+      <c r="E19" s="5" t="n">
         <v>6643.52</v>
       </c>
       <c r="F19" s="4" t="n">
@@ -17339,19 +17510,19 @@
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="6" t="n">
+      <c r="A20" s="7" t="n">
         <v>45589</v>
       </c>
-      <c r="B20" s="3" t="n">
+      <c r="B20" s="5" t="n">
         <v>1564.22</v>
       </c>
-      <c r="C20" s="3" t="n">
+      <c r="C20" s="5" t="n">
         <v>5.75</v>
       </c>
-      <c r="D20" s="3" t="n">
+      <c r="D20" s="5" t="n">
         <v>2.4</v>
       </c>
-      <c r="E20" s="3" t="n">
+      <c r="E20" s="5" t="n">
         <v>6725.8</v>
       </c>
       <c r="F20" s="4" t="n">
@@ -17376,19 +17547,19 @@
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A21" s="6" t="n">
+      <c r="A21" s="7" t="n">
         <v>45595</v>
       </c>
-      <c r="B21" s="3" t="n">
+      <c r="B21" s="5" t="n">
         <v>1549.32</v>
       </c>
-      <c r="C21" s="3" t="n">
+      <c r="C21" s="5" t="n">
         <v>5.76</v>
       </c>
-      <c r="D21" s="3" t="n">
+      <c r="D21" s="5" t="n">
         <v>2.5</v>
       </c>
-      <c r="E21" s="3" t="n">
+      <c r="E21" s="5" t="n">
         <v>6550.32</v>
       </c>
       <c r="F21" s="4" t="n">
@@ -17413,19 +17584,19 @@
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A22" s="6" t="n">
+      <c r="A22" s="7" t="n">
         <v>45604</v>
       </c>
-      <c r="B22" s="3" t="n">
+      <c r="B22" s="5" t="n">
         <v>1516.75</v>
       </c>
-      <c r="C22" s="3" t="n">
+      <c r="C22" s="5" t="n">
         <v>5.8</v>
       </c>
-      <c r="D22" s="3" t="n">
+      <c r="D22" s="5" t="n">
         <v>2.35</v>
       </c>
-      <c r="E22" s="3" t="n">
+      <c r="E22" s="5" t="n">
         <v>6519.72</v>
       </c>
       <c r="F22" s="4" t="n">
@@ -17450,19 +17621,19 @@
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A23" s="6" t="n">
+      <c r="A23" s="7" t="n">
         <v>45616</v>
       </c>
-      <c r="B23" s="3" t="n">
+      <c r="B23" s="5" t="n">
         <v>1502.94</v>
       </c>
-      <c r="C23" s="3" t="n">
+      <c r="C23" s="5" t="n">
         <v>5.91</v>
       </c>
-      <c r="D23" s="3" t="n">
+      <c r="D23" s="5" t="n">
         <v>2.41</v>
       </c>
-      <c r="E23" s="3" t="n">
+      <c r="E23" s="5" t="n">
         <v>6576.33</v>
       </c>
       <c r="F23" s="4" t="n">
@@ -17487,19 +17658,19 @@
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A24" s="6" t="n">
+      <c r="A24" s="7" t="n">
         <v>45625</v>
       </c>
-      <c r="B24" s="3" t="n">
+      <c r="B24" s="5" t="n">
         <v>1623.33</v>
       </c>
-      <c r="C24" s="3" t="n">
+      <c r="C24" s="5" t="n">
         <v>5.68</v>
       </c>
-      <c r="D24" s="3" t="n">
+      <c r="D24" s="5" t="n">
         <v>2.18</v>
       </c>
-      <c r="E24" s="3" t="n">
+      <c r="E24" s="5" t="n">
         <v>6576.6</v>
       </c>
       <c r="F24" s="4" t="n">
@@ -17524,19 +17695,19 @@
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A25" s="6" t="n">
+      <c r="A25" s="7" t="n">
         <v>45632</v>
       </c>
-      <c r="B25" s="3" t="n">
+      <c r="B25" s="5" t="n">
         <v>1646.03</v>
       </c>
-      <c r="C25" s="3" t="n">
+      <c r="C25" s="5" t="n">
         <v>5.58</v>
       </c>
-      <c r="D25" s="3" t="n">
+      <c r="D25" s="5" t="n">
         <v>2.18</v>
       </c>
-      <c r="E25" s="3" t="n">
+      <c r="E25" s="5" t="n">
         <v>6648.65</v>
       </c>
       <c r="F25" s="4" t="n">
@@ -17561,19 +17732,19 @@
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A26" s="6" t="n">
+      <c r="A26" s="7" t="n">
         <v>45645</v>
       </c>
-      <c r="B26" s="3" t="n">
+      <c r="B26" s="5" t="n">
         <v>1672</v>
       </c>
-      <c r="C26" s="3" t="n">
+      <c r="C26" s="5" t="n">
         <v>5.88</v>
       </c>
-      <c r="D26" s="3" t="n">
+      <c r="D26" s="5" t="n">
         <v>2.4</v>
       </c>
-      <c r="E26" s="3" t="n">
+      <c r="E26" s="5" t="n">
         <v>6699.84</v>
       </c>
       <c r="F26" s="4" t="n">
@@ -17598,19 +17769,19 @@
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A27" s="6" t="n">
+      <c r="A27" s="7" t="n">
         <v>45653</v>
       </c>
-      <c r="B27" s="3" t="n">
+      <c r="B27" s="5" t="n">
         <v>1630.1</v>
       </c>
-      <c r="C27" s="3" t="n">
+      <c r="C27" s="5" t="n">
         <v>5.99</v>
       </c>
-      <c r="D27" s="3" t="n">
+      <c r="D27" s="5" t="n">
         <v>2.65</v>
       </c>
-      <c r="E27" s="3" t="n">
+      <c r="E27" s="5" t="n">
         <v>6703.27</v>
       </c>
       <c r="F27" s="4" t="n">
@@ -17635,19 +17806,19 @@
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A28" s="6" t="n">
+      <c r="A28" s="7" t="n">
         <v>45659</v>
       </c>
-      <c r="B28" s="3" t="n">
+      <c r="B28" s="5" t="n">
         <v>1630</v>
       </c>
-      <c r="C28" s="3" t="n">
+      <c r="C28" s="5" t="n">
         <v>5.93</v>
       </c>
-      <c r="D28" s="3" t="n">
+      <c r="D28" s="5" t="n">
         <v>2.58</v>
       </c>
-      <c r="E28" s="3" t="n">
+      <c r="E28" s="5" t="n">
         <v>6681.92</v>
       </c>
       <c r="F28" s="4" t="n">
@@ -17672,19 +17843,19 @@
       </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A29" s="6" t="n">
+      <c r="A29" s="7" t="n">
         <v>45666</v>
       </c>
-      <c r="B29" s="3" t="n">
+      <c r="B29" s="5" t="n">
         <v>1620</v>
       </c>
-      <c r="C29" s="3" t="n">
+      <c r="C29" s="5" t="n">
         <v>6.05</v>
       </c>
-      <c r="D29" s="3" t="n">
+      <c r="D29" s="5" t="n">
         <v>2.75</v>
       </c>
-      <c r="E29" s="3" t="n">
+      <c r="E29" s="5" t="n">
         <v>6802.58</v>
       </c>
       <c r="F29" s="4" t="n">
@@ -17709,19 +17880,19 @@
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A30" s="6" t="n">
+      <c r="A30" s="7" t="n">
         <v>45674</v>
       </c>
-      <c r="B30" s="3" t="n">
+      <c r="B30" s="5" t="n">
         <v>1601</v>
       </c>
-      <c r="C30" s="3" t="n">
+      <c r="C30" s="5" t="n">
         <v>5.93</v>
       </c>
-      <c r="D30" s="3" t="n">
+      <c r="D30" s="5" t="n">
         <v>2.64</v>
       </c>
-      <c r="E30" s="3" t="n">
+      <c r="E30" s="5" t="n">
         <v>6958.79</v>
       </c>
       <c r="F30" s="4" t="n">
@@ -17746,19 +17917,19 @@
       </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A31" s="6" t="n">
+      <c r="A31" s="7" t="n">
         <v>45681</v>
       </c>
-      <c r="B31" s="3" t="n">
+      <c r="B31" s="5" t="n">
         <v>1684.8</v>
       </c>
-      <c r="C31" s="3" t="n">
+      <c r="C31" s="5" t="n">
         <v>6.01</v>
       </c>
-      <c r="D31" s="3" t="n">
+      <c r="D31" s="5" t="n">
         <v>2.38</v>
       </c>
-      <c r="E31" s="3" t="n">
+      <c r="E31" s="5" t="n">
         <v>7068.67</v>
       </c>
       <c r="F31" s="4" t="n">
@@ -17783,19 +17954,19 @@
       </c>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A32" s="6" t="n">
+      <c r="A32" s="7" t="n">
         <v>45688</v>
       </c>
-      <c r="B32" s="3" t="n">
+      <c r="B32" s="5" t="n">
         <v>1759.9</v>
       </c>
-      <c r="C32" s="3" t="n">
+      <c r="C32" s="5" t="n">
         <v>6.03</v>
       </c>
-      <c r="D32" s="3" t="n">
+      <c r="D32" s="5" t="n">
         <v>2.55</v>
       </c>
-      <c r="E32" s="3" t="n">
+      <c r="E32" s="5" t="n">
         <v>7199.59</v>
       </c>
       <c r="F32" s="4" t="n">
@@ -17820,19 +17991,19 @@
       </c>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A33" s="6" t="n">
+      <c r="A33" s="7" t="n">
         <v>45694</v>
       </c>
-      <c r="B33" s="3" t="n">
+      <c r="B33" s="5" t="n">
         <v>1805</v>
       </c>
-      <c r="C33" s="3" t="n">
+      <c r="C33" s="5" t="n">
         <v>5.98</v>
       </c>
-      <c r="D33" s="3" t="n">
+      <c r="D33" s="5" t="n">
         <v>2.49</v>
       </c>
-      <c r="E33" s="3" t="n">
+      <c r="E33" s="5" t="n">
         <v>7301.44</v>
       </c>
       <c r="F33" s="4" t="n">
@@ -17857,19 +18028,19 @@
       </c>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A34" s="6" t="n">
+      <c r="A34" s="7" t="n">
         <v>45699</v>
       </c>
-      <c r="B34" s="3" t="n">
+      <c r="B34" s="5" t="n">
         <v>1791</v>
       </c>
-      <c r="C34" s="3" t="n">
+      <c r="C34" s="5" t="n">
         <v>6</v>
       </c>
-      <c r="D34" s="3" t="n">
+      <c r="D34" s="5" t="n">
         <v>2.45</v>
       </c>
-      <c r="E34" s="3" t="n">
+      <c r="E34" s="5" t="n">
         <v>7278.04</v>
       </c>
       <c r="F34" s="4" t="n">
@@ -17894,19 +18065,19 @@
       </c>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A35" s="6" t="n">
+      <c r="A35" s="7" t="n">
         <v>45708</v>
       </c>
-      <c r="B35" s="3" t="n">
+      <c r="B35" s="5" t="n">
         <v>1881.3</v>
       </c>
-      <c r="C35" s="3" t="n">
+      <c r="C35" s="5" t="n">
         <v>6.1</v>
       </c>
-      <c r="D35" s="3" t="n">
+      <c r="D35" s="5" t="n">
         <v>2.6</v>
       </c>
-      <c r="E35" s="3" t="n">
+      <c r="E35" s="5" t="n">
         <v>7322.48</v>
       </c>
       <c r="F35" s="4" t="n">
@@ -17931,19 +18102,19 @@
       </c>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A36" s="6" t="n">
+      <c r="A36" s="7" t="n">
         <v>45716</v>
       </c>
-      <c r="B36" s="3" t="n">
+      <c r="B36" s="5" t="n">
         <v>1900</v>
       </c>
-      <c r="C36" s="3" t="n">
+      <c r="C36" s="5" t="n">
         <v>5.94</v>
       </c>
-      <c r="D36" s="3" t="n">
+      <c r="D36" s="5" t="n">
         <v>2.65</v>
       </c>
-      <c r="E36" s="3" t="n">
+      <c r="E36" s="5" t="n">
         <v>7332.12</v>
       </c>
       <c r="F36" s="4" t="n">
@@ -17968,19 +18139,19 @@
       </c>
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A37" s="6" t="n">
+      <c r="A37" s="7" t="n">
         <v>45720</v>
       </c>
-      <c r="B37" s="3" t="n">
+      <c r="B37" s="5" t="n">
         <v>1855</v>
       </c>
-      <c r="C37" s="3" t="n">
+      <c r="C37" s="5" t="n">
         <v>5.86</v>
       </c>
-      <c r="D37" s="3" t="n">
+      <c r="D37" s="5" t="n">
         <v>2.58</v>
       </c>
-      <c r="E37" s="3" t="n">
+      <c r="E37" s="5" t="n">
         <v>7313.89</v>
       </c>
       <c r="F37" s="4" t="n">
@@ -18005,19 +18176,19 @@
       </c>
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A38" s="6" t="n">
+      <c r="A38" s="7" t="n">
         <v>45730</v>
       </c>
-      <c r="B38" s="3" t="n">
+      <c r="B38" s="5" t="n">
         <v>1940</v>
       </c>
-      <c r="C38" s="3" t="n">
+      <c r="C38" s="5" t="n">
         <v>5.76</v>
       </c>
-      <c r="D38" s="3" t="n">
+      <c r="D38" s="5" t="n">
         <v>2.52</v>
       </c>
-      <c r="E38" s="3" t="n">
+      <c r="E38" s="5" t="n">
         <v>7509</v>
       </c>
       <c r="F38" s="4" t="n">
@@ -18042,19 +18213,19 @@
       </c>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A39" s="6" t="n">
+      <c r="A39" s="7" t="n">
         <v>45735</v>
       </c>
-      <c r="B39" s="3" t="n">
+      <c r="B39" s="5" t="n">
         <v>1970.1</v>
       </c>
-      <c r="C39" s="3" t="n">
+      <c r="C39" s="5" t="n">
         <v>5.76</v>
       </c>
-      <c r="D39" s="3" t="n">
+      <c r="D39" s="5" t="n">
         <v>2.54</v>
       </c>
-      <c r="E39" s="3" t="n">
+      <c r="E39" s="5" t="n">
         <v>7594.95</v>
       </c>
       <c r="F39" s="4" t="n">
@@ -18079,19 +18250,19 @@
       </c>
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A40" s="6" t="n">
+      <c r="A40" s="7" t="n">
         <v>45744</v>
       </c>
-      <c r="B40" s="3" t="n">
+      <c r="B40" s="5" t="n">
         <v>1970</v>
       </c>
-      <c r="C40" s="3" t="n">
+      <c r="C40" s="5" t="n">
         <v>5.85</v>
       </c>
-      <c r="D40" s="3" t="n">
+      <c r="D40" s="5" t="n">
         <v>2.63</v>
       </c>
-      <c r="E40" s="3" t="n">
+      <c r="E40" s="5" t="n">
         <v>7694.49</v>
       </c>
       <c r="F40" s="4" t="n">
@@ -18116,19 +18287,19 @@
       </c>
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A41" s="6" t="n">
+      <c r="A41" s="7" t="n">
         <v>45751</v>
       </c>
-      <c r="B41" s="3" t="n">
+      <c r="B41" s="5" t="n">
         <v>2000</v>
       </c>
-      <c r="C41" s="3" t="n">
+      <c r="C41" s="5" t="n">
         <v>5.55</v>
       </c>
-      <c r="D41" s="3" t="n">
+      <c r="D41" s="5" t="n">
         <v>2.28</v>
       </c>
-      <c r="E41" s="3" t="n">
+      <c r="E41" s="5" t="n">
         <v>7504.21</v>
       </c>
       <c r="F41" s="4" t="n">
@@ -18153,19 +18324,19 @@
       </c>
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A42" s="6" t="n">
+      <c r="A42" s="7" t="n">
         <v>45758</v>
       </c>
-      <c r="B42" s="3" t="n">
+      <c r="B42" s="5" t="n">
         <v>2049.9</v>
       </c>
-      <c r="C42" s="3" t="n">
+      <c r="C42" s="5" t="n">
         <v>5.68</v>
       </c>
-      <c r="D42" s="3" t="n">
+      <c r="D42" s="5" t="n">
         <v>2.42</v>
       </c>
-      <c r="E42" s="3" t="n">
+      <c r="E42" s="5" t="n">
         <v>7430.69</v>
       </c>
       <c r="F42" s="4" t="n">
@@ -18190,19 +18361,19 @@
       </c>
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A43" s="6" t="n">
+      <c r="A43" s="7" t="n">
         <v>45764</v>
       </c>
-      <c r="B43" s="3" t="n">
+      <c r="B43" s="5" t="n">
         <v>2179.9</v>
       </c>
-      <c r="C43" s="3" t="n">
+      <c r="C43" s="5" t="n">
         <v>5.58</v>
       </c>
-      <c r="D43" s="3" t="n">
+      <c r="D43" s="5" t="n">
         <v>2.49</v>
       </c>
-      <c r="E43" s="3" t="n">
+      <c r="E43" s="5" t="n">
         <v>7815.25</v>
       </c>
       <c r="F43" s="4" t="n">
@@ -18227,19 +18398,19 @@
       </c>
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A44" s="6" t="n">
+      <c r="A44" s="7" t="n">
         <v>45772</v>
       </c>
-      <c r="B44" s="3" t="n">
+      <c r="B44" s="5" t="n">
         <v>2200</v>
       </c>
-      <c r="C44" s="3" t="n">
+      <c r="C44" s="5" t="n">
         <v>5.71</v>
       </c>
-      <c r="D44" s="3" t="n">
+      <c r="D44" s="5" t="n">
         <v>2.48</v>
       </c>
-      <c r="E44" s="3" t="n">
+      <c r="E44" s="5" t="n">
         <v>7991.62</v>
       </c>
       <c r="F44" s="4" t="n">
@@ -18264,19 +18435,19 @@
       </c>
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A45" s="6" t="n">
+      <c r="A45" s="7" t="n">
         <v>45777</v>
       </c>
-      <c r="B45" s="3" t="n">
+      <c r="B45" s="5" t="n">
         <v>2225</v>
       </c>
-      <c r="C45" s="3" t="n">
+      <c r="C45" s="5" t="n">
         <v>5.7</v>
       </c>
-      <c r="D45" s="3" t="n">
+      <c r="D45" s="5" t="n">
         <v>2.45</v>
       </c>
-      <c r="E45" s="3" t="n">
+      <c r="E45" s="5" t="n">
         <v>8041.14</v>
       </c>
       <c r="F45" s="4" t="n">
@@ -18301,19 +18472,19 @@
       </c>
     </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A46" s="6" t="n">
+      <c r="A46" s="7" t="n">
         <v>45784</v>
       </c>
-      <c r="B46" s="3" t="n">
+      <c r="B46" s="5" t="n">
         <v>2240</v>
       </c>
-      <c r="C46" s="3" t="n">
+      <c r="C46" s="5" t="n">
         <v>5.78</v>
       </c>
-      <c r="D46" s="3" t="n">
+      <c r="D46" s="5" t="n">
         <v>2.53</v>
       </c>
-      <c r="E46" s="3" t="n">
+      <c r="E46" s="5" t="n">
         <v>8173.81</v>
       </c>
       <c r="F46" s="4" t="n">
@@ -18338,19 +18509,19 @@
       </c>
     </row>
     <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A47" s="6" t="n">
+      <c r="A47" s="7" t="n">
         <v>45793</v>
       </c>
-      <c r="B47" s="3" t="n">
+      <c r="B47" s="5" t="n">
         <v>2177</v>
       </c>
-      <c r="C47" s="3" t="n">
+      <c r="C47" s="5" t="n">
         <v>5.75</v>
       </c>
-      <c r="D47" s="3" t="n">
+      <c r="D47" s="5" t="n">
         <v>2.56</v>
       </c>
-      <c r="E47" s="3" t="n">
+      <c r="E47" s="5" t="n">
         <v>8386.16</v>
       </c>
       <c r="F47" s="4" t="n">
@@ -18375,19 +18546,19 @@
       </c>
     </row>
     <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A48" s="6" t="n">
+      <c r="A48" s="7" t="n">
         <v>45799</v>
       </c>
-      <c r="B48" s="3" t="n">
+      <c r="B48" s="5" t="n">
         <v>2225.5</v>
       </c>
-      <c r="C48" s="3" t="n">
+      <c r="C48" s="5" t="n">
         <v>5.8</v>
       </c>
-      <c r="D48" s="3" t="n">
+      <c r="D48" s="5" t="n">
         <v>2.58</v>
       </c>
-      <c r="E48" s="3" t="n">
+      <c r="E48" s="5" t="n">
         <v>8367.62</v>
       </c>
       <c r="F48" s="4" t="n">
@@ -18412,19 +18583,19 @@
       </c>
     </row>
     <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A49" s="6" t="n">
+      <c r="A49" s="7" t="n">
         <v>45807</v>
       </c>
-      <c r="B49" s="3" t="n">
+      <c r="B49" s="5" t="n">
         <v>2060</v>
       </c>
-      <c r="C49" s="3" t="n">
+      <c r="C49" s="5" t="n">
         <v>5.77</v>
       </c>
-      <c r="D49" s="3" t="n">
+      <c r="D49" s="5" t="n">
         <v>2.57</v>
       </c>
-      <c r="E49" s="3" t="n">
+      <c r="E49" s="5" t="n">
         <v>8047.51</v>
       </c>
       <c r="F49" s="4" t="n">
@@ -18449,19 +18620,19 @@
       </c>
     </row>
     <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A50" s="6" t="n">
+      <c r="A50" s="7" t="n">
         <v>45813</v>
       </c>
-      <c r="B50" s="3" t="n">
+      <c r="B50" s="5" t="n">
         <v>2070</v>
       </c>
-      <c r="C50" s="3" t="n">
+      <c r="C50" s="5" t="n">
         <v>5.75</v>
       </c>
-      <c r="D50" s="3" t="n">
+      <c r="D50" s="5" t="n">
         <v>2.6</v>
       </c>
-      <c r="E50" s="3" t="n">
+      <c r="E50" s="5" t="n">
         <v>8145.59</v>
       </c>
       <c r="F50" s="4" t="n">
@@ -18486,19 +18657,19 @@
       </c>
     </row>
     <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A51" s="6" t="n">
+      <c r="A51" s="7" t="n">
         <v>45821</v>
       </c>
-      <c r="B51" s="3" t="n">
+      <c r="B51" s="5" t="n">
         <v>2080</v>
       </c>
-      <c r="C51" s="3" t="n">
+      <c r="C51" s="5" t="n">
         <v>5.76</v>
       </c>
-      <c r="D51" s="3" t="n">
+      <c r="D51" s="5" t="n">
         <v>2.61</v>
       </c>
-      <c r="E51" s="3" t="n">
+      <c r="E51" s="5" t="n">
         <v>8209.92</v>
       </c>
       <c r="F51" s="4" t="n">
@@ -18523,19 +18694,19 @@
       </c>
     </row>
     <row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A52" s="6" t="n">
+      <c r="A52" s="7" t="n">
         <v>45824</v>
       </c>
-      <c r="B52" s="3" t="n">
+      <c r="B52" s="5" t="n">
         <v>2070.6</v>
       </c>
-      <c r="C52" s="3" t="n">
+      <c r="C52" s="5" t="n">
         <v>5.73</v>
       </c>
-      <c r="D52" s="3" t="n">
+      <c r="D52" s="5" t="n">
         <v>2.6</v>
       </c>
-      <c r="E52" s="3" t="n">
+      <c r="E52" s="5" t="n">
         <v>8165.29</v>
       </c>
       <c r="F52" s="4" t="n">
@@ -18560,19 +18731,19 @@
       </c>
     </row>
     <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A53" s="6" t="n">
+      <c r="A53" s="7" t="n">
         <v>45835</v>
       </c>
-      <c r="B53" s="3" t="n">
+      <c r="B53" s="5" t="n">
         <v>2050.1</v>
       </c>
-      <c r="C53" s="3" t="n">
+      <c r="C53" s="5" t="n">
         <v>5.68</v>
       </c>
-      <c r="D53" s="3" t="n">
+      <c r="D53" s="5" t="n">
         <v>2.69</v>
       </c>
-      <c r="E53" s="3" t="n">
+      <c r="E53" s="5" t="n">
         <v>8213.08</v>
       </c>
       <c r="F53" s="4" t="n">
@@ -18597,19 +18768,19 @@
       </c>
     </row>
     <row r="54" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A54" s="6" t="n">
+      <c r="A54" s="7" t="n">
         <v>45841</v>
       </c>
-      <c r="B54" s="3" t="n">
+      <c r="B54" s="5" t="n">
         <v>2080</v>
       </c>
-      <c r="C54" s="3" t="n">
+      <c r="C54" s="5" t="n">
         <v>5.67</v>
       </c>
-      <c r="D54" s="3" t="n">
+      <c r="D54" s="5" t="n">
         <v>2.65</v>
       </c>
-      <c r="E54" s="3" t="n">
+      <c r="E54" s="5" t="n">
         <v>8290.26</v>
       </c>
       <c r="F54" s="4" t="n">
@@ -18634,19 +18805,19 @@
       </c>
     </row>
     <row r="55" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A55" s="6" t="n">
+      <c r="A55" s="7" t="n">
         <v>45849</v>
       </c>
-      <c r="B55" s="3" t="n">
+      <c r="B55" s="5" t="n">
         <v>2190</v>
       </c>
-      <c r="C55" s="3" t="n">
+      <c r="C55" s="5" t="n">
         <v>5.61</v>
       </c>
-      <c r="D55" s="3" t="n">
+      <c r="D55" s="5" t="n">
         <v>2.68</v>
       </c>
-      <c r="E55" s="3" t="n">
+      <c r="E55" s="5" t="n">
         <v>8231.92</v>
       </c>
       <c r="F55" s="4" t="n">
@@ -18671,19 +18842,19 @@
       </c>
     </row>
     <row r="56" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A56" s="6" t="n">
+      <c r="A56" s="7" t="n">
         <v>45863</v>
       </c>
-      <c r="B56" s="3" t="n">
+      <c r="B56" s="5" t="n">
         <v>2065</v>
       </c>
-      <c r="C56" s="3" t="n">
+      <c r="C56" s="5" t="n">
         <v>5.6</v>
       </c>
-      <c r="D56" s="3" t="n">
+      <c r="D56" s="5" t="n">
         <v>2.52</v>
       </c>
-      <c r="E56" s="3" t="n">
+      <c r="E56" s="5" t="n">
         <v>8221.9</v>
       </c>
       <c r="F56" s="4" t="n">
@@ -18708,19 +18879,19 @@
       </c>
     </row>
     <row r="57" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A57" s="6" t="n">
+      <c r="A57" s="7" t="n">
         <v>45870</v>
       </c>
-      <c r="B57" s="3" t="n">
+      <c r="B57" s="5" t="n">
         <v>2124</v>
       </c>
-      <c r="C57" s="3" t="n">
+      <c r="C57" s="5" t="n">
         <v>5.6</v>
       </c>
-      <c r="D57" s="3" t="n">
+      <c r="D57" s="5" t="n">
         <v>2.45</v>
       </c>
-      <c r="E57" s="3" t="n">
+      <c r="E57" s="5" t="n">
         <v>8161.33</v>
       </c>
       <c r="F57" s="4" t="n">
@@ -18745,19 +18916,19 @@
       </c>
     </row>
     <row r="58" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A58" s="6" t="n">
+      <c r="A58" s="7" t="n">
         <v>45877</v>
       </c>
-      <c r="B58" s="3" t="n">
+      <c r="B58" s="5" t="n">
         <v>2164.9</v>
       </c>
-      <c r="C58" s="3" t="n">
+      <c r="C58" s="5" t="n">
         <v>5.63</v>
       </c>
-      <c r="D58" s="3" t="n">
+      <c r="D58" s="5" t="n">
         <v>2.36</v>
       </c>
-      <c r="E58" s="3" t="n">
+      <c r="E58" s="5" t="n">
         <v>8520.53</v>
       </c>
       <c r="F58" s="4" t="n">
@@ -18782,19 +18953,19 @@
       </c>
     </row>
     <row r="59" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A59" s="6" t="n">
+      <c r="A59" s="7" t="n">
         <v>45882</v>
       </c>
-      <c r="B59" s="3" t="n">
+      <c r="B59" s="5" t="n">
         <v>2228.1</v>
       </c>
-      <c r="C59" s="3" t="n">
+      <c r="C59" s="5" t="n">
         <v>5.59</v>
       </c>
-      <c r="D59" s="3" t="n">
+      <c r="D59" s="5" t="n">
         <v>2.37</v>
       </c>
-      <c r="E59" s="3" t="n">
+      <c r="E59" s="5" t="n">
         <v>8737.86</v>
       </c>
       <c r="F59" s="4" t="n">
@@ -18819,19 +18990,19 @@
       </c>
     </row>
     <row r="60" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A60" s="6" t="n">
+      <c r="A60" s="7" t="n">
         <v>45891</v>
       </c>
-      <c r="B60" s="3" t="n">
+      <c r="B60" s="5" t="n">
         <v>2242.2</v>
       </c>
-      <c r="C60" s="3" t="n">
+      <c r="C60" s="5" t="n">
         <v>5.57</v>
       </c>
-      <c r="D60" s="3" t="n">
+      <c r="D60" s="5" t="n">
         <v>2.49</v>
       </c>
-      <c r="E60" s="3" t="n">
+      <c r="E60" s="5" t="n">
         <v>8854.26</v>
       </c>
       <c r="F60" s="4" t="n">
@@ -18856,19 +19027,19 @@
       </c>
     </row>
     <row r="61" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A61" s="6" t="n">
+      <c r="A61" s="7" t="n">
         <v>45898</v>
       </c>
-      <c r="B61" s="3" t="n">
+      <c r="B61" s="5" t="n">
         <v>2270.1</v>
       </c>
-      <c r="C61" s="3" t="n">
+      <c r="C61" s="5" t="n">
         <v>5.63</v>
       </c>
-      <c r="D61" s="3" t="n">
+      <c r="D61" s="5" t="n">
         <v>2.48</v>
       </c>
-      <c r="E61" s="3" t="n">
+      <c r="E61" s="5" t="n">
         <v>8899.91</v>
       </c>
       <c r="F61" s="4" t="n">
@@ -18893,19 +19064,19 @@
       </c>
     </row>
     <row r="62" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A62" s="6" t="n">
+      <c r="A62" s="7" t="n">
         <v>45905</v>
       </c>
-      <c r="B62" s="3" t="n">
+      <c r="B62" s="5" t="n">
         <v>2454.11</v>
       </c>
-      <c r="C62" s="3" t="n">
+      <c r="C62" s="5" t="n">
         <v>5.67</v>
       </c>
-      <c r="D62" s="3" t="n">
+      <c r="D62" s="5" t="n">
         <v>2.41</v>
       </c>
-      <c r="E62" s="3" t="n">
+      <c r="E62" s="5" t="n">
         <v>9210.68</v>
       </c>
       <c r="F62" s="4" t="n">
@@ -18930,19 +19101,19 @@
       </c>
     </row>
     <row r="63" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A63" s="6" t="n">
+      <c r="A63" s="7" t="n">
         <v>45912</v>
       </c>
-      <c r="B63" s="3" t="n">
+      <c r="B63" s="5" t="n">
         <v>2515</v>
       </c>
-      <c r="C63" s="3" t="n">
+      <c r="C63" s="5" t="n">
         <v>5.62</v>
       </c>
-      <c r="D63" s="3" t="n">
+      <c r="D63" s="5" t="n">
         <v>2.42</v>
       </c>
-      <c r="E63" s="3" t="n">
+      <c r="E63" s="5" t="n">
         <v>8989.75</v>
       </c>
       <c r="F63" s="4" t="n">
@@ -18967,19 +19138,19 @@
       </c>
     </row>
     <row r="64" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A64" s="6" t="n">
+      <c r="A64" s="7" t="n">
         <v>45916</v>
       </c>
-      <c r="B64" s="3" t="n">
+      <c r="B64" s="5" t="n">
         <v>2580</v>
       </c>
-      <c r="C64" s="3" t="n">
+      <c r="C64" s="5" t="n">
         <v>5.6</v>
       </c>
-      <c r="D64" s="3" t="n">
+      <c r="D64" s="5" t="n">
         <v>2.41</v>
       </c>
-      <c r="E64" s="3" t="n">
+      <c r="E64" s="5" t="n">
         <v>9066.03</v>
       </c>
       <c r="F64" s="4" t="n">
@@ -19004,19 +19175,19 @@
       </c>
     </row>
     <row r="65" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A65" s="6" t="n">
+      <c r="A65" s="7" t="n">
         <v>45925</v>
       </c>
-      <c r="B65" s="3" t="n">
+      <c r="B65" s="5" t="n">
         <v>2585</v>
       </c>
-      <c r="C65" s="3" t="n">
+      <c r="C65" s="5" t="n">
         <v>5.58</v>
       </c>
-      <c r="D65" s="3" t="n">
+      <c r="D65" s="5" t="n">
         <v>2.4</v>
       </c>
-      <c r="E65" s="3" t="n">
+      <c r="E65" s="5" t="n">
         <v>9040.46</v>
       </c>
       <c r="F65" s="4" t="n">
@@ -19041,19 +19212,19 @@
       </c>
     </row>
     <row r="66" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A66" s="6" t="n">
+      <c r="A66" s="7" t="n">
         <v>45932</v>
       </c>
-      <c r="B66" s="3" t="n">
+      <c r="B66" s="5" t="n">
         <v>2580</v>
       </c>
-      <c r="C66" s="3" t="n">
+      <c r="C66" s="5" t="n">
         <v>5.63</v>
       </c>
-      <c r="D66" s="3" t="n">
+      <c r="D66" s="5" t="n">
         <v>2.34</v>
       </c>
-      <c r="E66" s="3" t="n">
+      <c r="E66" s="5" t="n">
         <v>8899.67</v>
       </c>
       <c r="F66" s="4" t="n">
@@ -19078,19 +19249,19 @@
       </c>
     </row>
     <row r="67" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A67" s="6" t="n">
+      <c r="A67" s="7" t="n">
         <v>45940</v>
       </c>
-      <c r="B67" s="3" t="n">
+      <c r="B67" s="5" t="n">
         <v>2537</v>
       </c>
-      <c r="C67" s="3" t="n">
+      <c r="C67" s="5" t="n">
         <v>5.58</v>
       </c>
-      <c r="D67" s="3" t="n">
+      <c r="D67" s="5" t="n">
         <v>2.34</v>
       </c>
-      <c r="E67" s="3" t="n">
+      <c r="E67" s="5" t="n">
         <v>8675.8</v>
       </c>
       <c r="F67" s="4" t="n">
@@ -19115,19 +19286,19 @@
       </c>
     </row>
     <row r="68" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A68" s="6" t="n">
+      <c r="A68" s="7" t="n">
         <v>45947</v>
       </c>
-      <c r="B68" s="3" t="n">
+      <c r="B68" s="5" t="n">
         <v>2689.9</v>
       </c>
-      <c r="C68" s="3" t="n">
+      <c r="C68" s="5" t="n">
         <v>5.57</v>
       </c>
-      <c r="D68" s="3" t="n">
+      <c r="D68" s="5" t="n">
         <v>2.36</v>
       </c>
-      <c r="E68" s="3" t="n">
+      <c r="E68" s="5" t="n">
         <v>9129.98</v>
       </c>
       <c r="F68" s="4" t="n">
@@ -19152,19 +19323,19 @@
       </c>
     </row>
     <row r="69" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A69" s="6" t="n">
+      <c r="A69" s="7" t="n">
         <v>45954</v>
       </c>
-      <c r="B69" s="3" t="n">
+      <c r="B69" s="5" t="n">
         <v>2730</v>
       </c>
-      <c r="C69" s="3" t="n">
+      <c r="C69" s="5" t="n">
         <v>5.55</v>
       </c>
-      <c r="D69" s="3" t="n">
+      <c r="D69" s="5" t="n">
         <v>2.38</v>
       </c>
-      <c r="E69" s="3" t="n">
+      <c r="E69" s="5" t="n">
         <v>9184.41</v>
       </c>
       <c r="F69" s="4" t="n">
@@ -19189,19 +19360,19 @@
       </c>
     </row>
     <row r="70" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A70" s="6" t="n">
+      <c r="A70" s="7" t="n">
         <v>45960</v>
       </c>
-      <c r="B70" s="3" t="n">
+      <c r="B70" s="5" t="n">
         <v>2655</v>
       </c>
-      <c r="C70" s="3" t="n">
+      <c r="C70" s="5" t="n">
         <v>5.56</v>
       </c>
-      <c r="D70" s="3" t="n">
+      <c r="D70" s="5" t="n">
         <v>2.37</v>
       </c>
-      <c r="E70" s="3" t="n">
+      <c r="E70" s="5" t="n">
         <v>9428.89</v>
       </c>
       <c r="F70" s="4" t="n">
@@ -19226,19 +19397,19 @@
       </c>
     </row>
     <row r="71" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A71" s="6" t="n">
+      <c r="A71" s="7" t="n">
         <v>45968</v>
       </c>
-      <c r="B71" s="3" t="n">
+      <c r="B71" s="5" t="n">
         <v>2955</v>
       </c>
-      <c r="C71" s="3" t="n">
+      <c r="C71" s="5" t="n">
         <v>5.52</v>
       </c>
-      <c r="D71" s="3" t="n">
+      <c r="D71" s="5" t="n">
         <v>2.37</v>
       </c>
-      <c r="E71" s="3" t="n">
+      <c r="E71" s="5" t="n">
         <v>9605.06</v>
       </c>
       <c r="F71" s="4" t="n">
@@ -19263,19 +19434,19 @@
       </c>
     </row>
     <row r="72" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A72" s="6" t="n">
+      <c r="A72" s="7" t="n">
         <v>45975</v>
       </c>
-      <c r="B72" s="3" t="n">
+      <c r="B72" s="5" t="n">
         <v>2977</v>
       </c>
-      <c r="C72" s="3" t="n">
+      <c r="C72" s="5" t="n">
         <v>5.38</v>
       </c>
-      <c r="D72" s="3" t="n">
+      <c r="D72" s="5" t="n">
         <v>2.36</v>
       </c>
-      <c r="E72" s="3" t="n">
+      <c r="E72" s="5" t="n">
         <v>9603.02</v>
       </c>
       <c r="F72" s="4" t="n">
@@ -19300,19 +19471,19 @@
       </c>
     </row>
     <row r="73" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A73" s="6" t="n">
+      <c r="A73" s="7" t="n">
         <v>45981</v>
       </c>
-      <c r="B73" s="3" t="n">
+      <c r="B73" s="5" t="n">
         <v>3015</v>
       </c>
-      <c r="C73" s="3" t="n">
+      <c r="C73" s="5" t="n">
         <v>5.35</v>
       </c>
-      <c r="D73" s="3" t="n">
+      <c r="D73" s="5" t="n">
         <v>2.33</v>
       </c>
-      <c r="E73" s="3" t="n">
+      <c r="E73" s="5" t="n">
         <v>9802.08</v>
       </c>
       <c r="F73" s="4" t="n">
@@ -19337,19 +19508,19 @@
       </c>
     </row>
     <row r="74" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A74" s="6" t="n">
+      <c r="A74" s="7" t="n">
         <v>45986</v>
       </c>
-      <c r="B74" s="3" t="n">
+      <c r="B74" s="5" t="n">
         <v>3110</v>
       </c>
-      <c r="C74" s="3" t="n">
+      <c r="C74" s="5" t="n">
         <v>5.31</v>
       </c>
-      <c r="D74" s="3" t="n">
+      <c r="D74" s="5" t="n">
         <v>2.31</v>
       </c>
-      <c r="E74" s="3" t="n">
+      <c r="E74" s="5" t="n">
         <v>9950.81</v>
       </c>
       <c r="F74" s="4" t="n">
@@ -19374,19 +19545,19 @@
       </c>
     </row>
     <row r="75" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A75" s="6" t="n">
+      <c r="A75" s="7" t="n">
         <v>45996</v>
       </c>
-      <c r="B75" s="3" t="n">
+      <c r="B75" s="5" t="n">
         <v>3243</v>
       </c>
-      <c r="C75" s="3" t="n">
+      <c r="C75" s="5" t="n">
         <v>5.32</v>
       </c>
-      <c r="D75" s="3" t="n">
+      <c r="D75" s="5" t="n">
         <v>2.32</v>
       </c>
-      <c r="E75" s="3" t="n">
+      <c r="E75" s="5" t="n">
         <v>10222.61</v>
       </c>
       <c r="F75" s="4" t="n">
@@ -19411,19 +19582,19 @@
       </c>
     </row>
     <row r="76" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A76" s="6" t="n">
+      <c r="A76" s="7" t="n">
         <v>46003</v>
       </c>
-      <c r="B76" s="3" t="n">
+      <c r="B76" s="5" t="n">
         <v>3275</v>
       </c>
-      <c r="C76" s="3" t="n">
+      <c r="C76" s="5" t="n">
         <v>5.32</v>
       </c>
-      <c r="D76" s="3" t="n">
+      <c r="D76" s="5" t="n">
         <v>2.34</v>
       </c>
-      <c r="E76" s="3" t="n">
+      <c r="E76" s="5" t="n">
         <v>10400.01</v>
       </c>
       <c r="F76" s="4" t="n">
@@ -19448,19 +19619,19 @@
       </c>
     </row>
     <row r="77" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A77" s="6" t="n">
+      <c r="A77" s="7" t="n">
         <v>46009</v>
       </c>
-      <c r="B77" s="3" t="n">
+      <c r="B77" s="5" t="n">
         <v>3140</v>
       </c>
-      <c r="C77" s="3" t="n">
+      <c r="C77" s="5" t="n">
         <v>5.39</v>
       </c>
-      <c r="D77" s="3" t="n">
+      <c r="D77" s="5" t="n">
         <v>2.32</v>
       </c>
-      <c r="E77" s="3" t="n">
+      <c r="E77" s="5" t="n">
         <v>10194.26</v>
       </c>
       <c r="F77" s="4" t="n">
@@ -19485,19 +19656,19 @@
       </c>
     </row>
     <row r="78" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A78" s="6" t="n">
+      <c r="A78" s="7" t="n">
         <v>46017</v>
       </c>
-      <c r="B78" s="3" t="n">
+      <c r="B78" s="5" t="n">
         <v>3125</v>
       </c>
-      <c r="C78" s="3" t="n">
+      <c r="C78" s="5" t="n">
         <v>5.4</v>
       </c>
-      <c r="D78" s="3" t="n">
+      <c r="D78" s="5" t="n">
         <v>2.34</v>
       </c>
-      <c r="E78" s="3" t="n">
+      <c r="E78" s="5" t="n">
         <v>10483.15</v>
       </c>
       <c r="F78" s="4" t="n">
@@ -19522,19 +19693,19 @@
       </c>
     </row>
     <row r="79" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A79" s="6" t="n">
+      <c r="A79" s="7" t="n">
         <v>46020</v>
       </c>
-      <c r="B79" s="3" t="n">
+      <c r="B79" s="5" t="n">
         <v>3194.9</v>
       </c>
-      <c r="C79" s="3" t="n">
+      <c r="C79" s="5" t="n">
         <v>5.41</v>
       </c>
-      <c r="D79" s="3" t="n">
+      <c r="D79" s="5" t="n">
         <v>2.33</v>
       </c>
-      <c r="E79" s="3" t="n">
+      <c r="E79" s="5" t="n">
         <v>10521.68</v>
       </c>
       <c r="F79" s="4" t="n">
@@ -19559,19 +19730,19 @@
       </c>
     </row>
     <row r="80" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A80" s="6" t="n">
+      <c r="A80" s="7" t="n">
         <v>46031</v>
       </c>
-      <c r="B80" s="3" t="n">
+      <c r="B80" s="5" t="n">
         <v>3395</v>
       </c>
-      <c r="C80" s="3" t="n">
+      <c r="C80" s="5" t="n">
         <v>5.31</v>
       </c>
-      <c r="D80" s="3" t="n">
+      <c r="D80" s="5" t="n">
         <v>2.31</v>
       </c>
-      <c r="E80" s="3" t="n">
+      <c r="E80" s="5" t="n">
         <v>10929.15</v>
       </c>
       <c r="F80" s="4" t="n">
@@ -19596,19 +19767,19 @@
       </c>
     </row>
     <row r="81" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A81" s="6" t="n">
+      <c r="A81" s="7" t="n">
         <v>46038</v>
       </c>
-      <c r="B81" s="3" t="n">
+      <c r="B81" s="5" t="n">
         <v>3650</v>
       </c>
-      <c r="C81" s="3" t="n">
+      <c r="C81" s="5" t="n">
         <v>5.34</v>
       </c>
-      <c r="D81" s="3" t="n">
+      <c r="D81" s="5" t="n">
         <v>2.32</v>
       </c>
-      <c r="E81" s="3" t="n">
+      <c r="E81" s="5" t="n">
         <v>11156.73</v>
       </c>
       <c r="F81" s="4" t="n">
@@ -19633,19 +19804,19 @@
       </c>
     </row>
     <row r="82" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A82" s="6" t="n">
+      <c r="A82" s="7" t="n">
         <v>46045</v>
       </c>
-      <c r="B82" s="3" t="n">
+      <c r="B82" s="5" t="n">
         <v>3800</v>
       </c>
-      <c r="C82" s="3" t="n">
+      <c r="C82" s="5" t="n">
         <v>5.34</v>
       </c>
-      <c r="D82" s="3" t="n">
+      <c r="D82" s="5" t="n">
         <v>2.33</v>
       </c>
-      <c r="E82" s="3" t="n">
+      <c r="E82" s="5" t="n">
         <v>11500.1</v>
       </c>
       <c r="F82" s="4" t="n">
@@ -19670,19 +19841,19 @@
       </c>
     </row>
     <row r="83" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A83" s="6" t="n">
+      <c r="A83" s="7" t="n">
         <v>46052</v>
       </c>
-      <c r="B83" s="3" t="n">
+      <c r="B83" s="5" t="n">
         <v>3800</v>
       </c>
-      <c r="C83" s="3" t="n">
+      <c r="C83" s="5" t="n">
         <v>5.34</v>
       </c>
-      <c r="D83" s="3" t="n">
+      <c r="D83" s="5" t="n">
         <v>2.33</v>
       </c>
-      <c r="E83" s="3" t="n">
+      <c r="E83" s="5" t="n">
         <v>11420.07</v>
       </c>
       <c r="F83" s="4" t="n">
@@ -19707,19 +19878,19 @@
       </c>
     </row>
     <row r="84" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A84" s="6" t="n">
+      <c r="A84" s="7" t="n">
         <v>46057</v>
       </c>
-      <c r="B84" s="3" t="n">
+      <c r="B84" s="5" t="n">
         <v>3889.9</v>
       </c>
-      <c r="C84" s="3" t="n">
+      <c r="C84" s="5" t="n">
         <v>5.34</v>
       </c>
-      <c r="D84" s="3" t="n">
+      <c r="D84" s="5" t="n">
         <v>2.36</v>
       </c>
-      <c r="E84" s="3" t="n">
+      <c r="E84" s="5" t="n">
         <v>11425.88</v>
       </c>
       <c r="F84" s="4" t="n">
@@ -19744,19 +19915,19 @@
       </c>
     </row>
     <row r="85" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A85" s="6" t="n">
+      <c r="A85" s="7" t="n">
         <v>46063</v>
       </c>
-      <c r="B85" s="3" t="n">
+      <c r="B85" s="5" t="n">
         <v>3725.5</v>
       </c>
-      <c r="C85" s="3" t="n">
+      <c r="C85" s="5" t="n">
         <v>5.31</v>
       </c>
-      <c r="D85" s="3" t="n">
+      <c r="D85" s="5" t="n">
         <v>2.31</v>
       </c>
-      <c r="E85" s="3" t="n">
+      <c r="E85" s="5" t="n">
         <v>11009.28</v>
       </c>
       <c r="F85" s="4" t="n">
@@ -19781,19 +19952,19 @@
       </c>
     </row>
     <row r="86" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A86" s="6" t="n">
+      <c r="A86" s="7" t="n">
         <v>46073</v>
       </c>
-      <c r="B86" s="3" t="n">
+      <c r="B86" s="5" t="n">
         <v>3905</v>
       </c>
-      <c r="C86" s="3" t="n">
+      <c r="C86" s="5" t="n">
         <v>5.28</v>
       </c>
-      <c r="D86" s="3" t="n">
+      <c r="D86" s="5" t="n">
         <v>2.3</v>
       </c>
-      <c r="E86" s="3" t="n">
+      <c r="E86" s="5" t="n">
         <v>10855.08</v>
       </c>
       <c r="F86" s="4" t="n">
@@ -19818,19 +19989,19 @@
       </c>
     </row>
     <row r="87" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A87" s="6" t="n">
+      <c r="A87" s="7" t="n">
         <v>46080</v>
       </c>
-      <c r="B87" s="3" t="n">
+      <c r="B87" s="5" t="n">
         <v>4080</v>
       </c>
-      <c r="C87" s="3" t="n">
+      <c r="C87" s="5" t="n">
         <v>5.25</v>
       </c>
-      <c r="D87" s="3" t="n">
+      <c r="D87" s="5" t="n">
         <v>2.29</v>
       </c>
-      <c r="E87" s="3" t="n">
+      <c r="E87" s="5" t="n">
         <v>10877.74</v>
       </c>
       <c r="F87" s="4" t="n">
@@ -19855,19 +20026,19 @@
       </c>
     </row>
     <row r="88" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A88" s="6" t="n">
+      <c r="A88" s="7" t="n">
         <v>46085</v>
       </c>
-      <c r="B88" s="3" t="n">
+      <c r="B88" s="5" t="n">
         <v>3920</v>
       </c>
-      <c r="C88" s="3" t="n">
+      <c r="C88" s="5" t="n">
         <v>5.3</v>
       </c>
-      <c r="D88" s="3" t="n">
+      <c r="D88" s="5" t="n">
         <v>2.24</v>
       </c>
-      <c r="E88" s="3" t="n">
+      <c r="E88" s="5" t="n">
         <v>10494.97</v>
       </c>
       <c r="F88" s="4" t="n">
@@ -19892,19 +20063,19 @@
       </c>
     </row>
     <row r="89" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A89" s="6" t="n">
+      <c r="A89" s="7" t="n">
         <v>46094</v>
       </c>
-      <c r="B89" s="3" t="n">
+      <c r="B89" s="5" t="n">
         <v>3824.9</v>
       </c>
-      <c r="C89" s="3" t="n">
+      <c r="C89" s="5" t="n">
         <v>5.46</v>
       </c>
-      <c r="D89" s="3" t="n">
+      <c r="D89" s="5" t="n">
         <v>2.15</v>
       </c>
-      <c r="E89" s="3" t="n">
+      <c r="E89" s="5" t="n">
         <v>10466.52</v>
       </c>
       <c r="F89" s="4" t="n">
@@ -19929,19 +20100,19 @@
       </c>
     </row>
     <row r="90" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A90" s="6" t="n">
+      <c r="A90" s="7" t="n">
         <v>46101</v>
       </c>
-      <c r="B90" s="3" t="n">
+      <c r="B90" s="5" t="n">
         <v>3900</v>
       </c>
-      <c r="C90" s="3" t="n">
+      <c r="C90" s="5" t="n">
         <v>5.66</v>
       </c>
-      <c r="D90" s="3" t="n">
+      <c r="D90" s="5" t="n">
         <v>2.25</v>
       </c>
-      <c r="E90" s="3" t="n">
+      <c r="E90" s="5" t="n">
         <v>10277.51</v>
       </c>
       <c r="F90" s="4" t="n">
@@ -19966,19 +20137,19 @@
       </c>
     </row>
     <row r="91" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A91" s="6" t="n">
+      <c r="A91" s="7" t="n">
         <v>46108</v>
       </c>
-      <c r="B91" s="3" t="n">
+      <c r="B91" s="5" t="n">
         <v>3810</v>
       </c>
-      <c r="C91" s="3" t="n">
+      <c r="C91" s="5" t="n">
         <v>5.69</v>
       </c>
-      <c r="D91" s="3" t="n">
+      <c r="D91" s="5" t="n">
         <v>2.16</v>
       </c>
-      <c r="E91" s="3" t="n">
+      <c r="E91" s="5" t="n">
         <v>10417.19</v>
       </c>
       <c r="F91" s="4" t="n">
@@ -20003,19 +20174,19 @@
       </c>
     </row>
     <row r="92" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A92" s="6" t="n">
+      <c r="A92" s="7" t="n">
         <v>46114</v>
       </c>
-      <c r="B92" s="3" t="n">
+      <c r="B92" s="5" t="n">
         <v>4000</v>
       </c>
-      <c r="C92" s="3" t="n">
+      <c r="C92" s="5" t="n">
         <v>5.56</v>
       </c>
-      <c r="D92" s="3" t="n">
+      <c r="D92" s="5" t="n">
         <v>2.1</v>
       </c>
-      <c r="E92" s="3" t="n">
+      <c r="E92" s="5" t="n">
         <v>10739.15</v>
       </c>
       <c r="F92" s="4" t="n">
@@ -20040,19 +20211,19 @@
       </c>
     </row>
     <row r="93" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A93" s="6" t="n">
+      <c r="A93" s="7" t="n">
         <v>46122</v>
       </c>
-      <c r="B93" s="3" t="n">
+      <c r="B93" s="5" t="n">
         <v>4150</v>
       </c>
-      <c r="C93" s="3" t="n">
+      <c r="C93" s="5" t="n">
         <v>5.46</v>
       </c>
-      <c r="D93" s="3" t="n">
+      <c r="D93" s="5" t="n">
         <v>2.1</v>
       </c>
-      <c r="E93" s="3" t="n">
+      <c r="E93" s="5" t="n">
         <v>11076.65</v>
       </c>
       <c r="F93" s="4" t="n">
@@ -20077,19 +20248,19 @@
       </c>
     </row>
     <row r="94" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A94" s="6" t="n">
+      <c r="A94" s="7" t="n">
         <v>46129</v>
       </c>
-      <c r="B94" s="3" t="n">
+      <c r="B94" s="5" t="n">
         <v>4585</v>
       </c>
-      <c r="C94" s="3" t="n">
+      <c r="C94" s="5" t="n">
         <v>5.34</v>
       </c>
-      <c r="D94" s="3" t="n">
+      <c r="D94" s="5" t="n">
         <v>2.15</v>
       </c>
-      <c r="E94" s="3" t="n">
+      <c r="E94" s="5" t="n">
         <v>11429.19</v>
       </c>
       <c r="F94" s="4" t="n">
@@ -20114,19 +20285,19 @@
       </c>
     </row>
     <row r="95" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A95" s="6" t="n">
+      <c r="A95" s="7" t="n">
         <v>46135</v>
       </c>
-      <c r="B95" s="3" t="n">
+      <c r="B95" s="5" t="n">
         <v>4414.7</v>
       </c>
-      <c r="C95" s="3" t="n">
+      <c r="C95" s="5" t="n">
         <v>5.46</v>
       </c>
-      <c r="D95" s="3" t="n">
+      <c r="D95" s="5" t="n">
         <v>2.18</v>
       </c>
-      <c r="E95" s="3" t="n">
+      <c r="E95" s="5" t="n">
         <v>10992.09</v>
       </c>
       <c r="F95" s="4" t="n">
@@ -20151,19 +20322,19 @@
       </c>
     </row>
     <row r="96" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A96" s="6" t="n">
+      <c r="A96" s="7" t="n">
         <v>46142</v>
       </c>
-      <c r="B96" s="3" t="n">
+      <c r="B96" s="5" t="n">
         <v>4469.9</v>
       </c>
-      <c r="C96" s="3" t="n">
+      <c r="C96" s="5" t="n">
         <v>5.61</v>
       </c>
-      <c r="D96" s="3" t="n">
+      <c r="D96" s="5" t="n">
         <v>2.21</v>
       </c>
-      <c r="E96" s="3" t="n">
+      <c r="E96" s="5" t="n">
         <v>10908.3</v>
       </c>
       <c r="F96" s="4" t="n">
@@ -20188,19 +20359,19 @@
       </c>
     </row>
     <row r="97" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A97" s="6" t="n">
+      <c r="A97" s="7" t="n">
         <v>46150</v>
       </c>
-      <c r="B97" s="3" t="n">
+      <c r="B97" s="5" t="n">
         <v>4009</v>
       </c>
-      <c r="C97" s="3" t="n">
+      <c r="C97" s="5" t="n">
         <v>5.56</v>
       </c>
-      <c r="D97" s="3" t="n">
+      <c r="D97" s="5" t="n">
         <v>2.25</v>
       </c>
-      <c r="E97" s="3" t="n">
+      <c r="E97" s="5" t="n">
         <v>10758.9</v>
       </c>
       <c r="F97" s="4" t="n">
@@ -20225,19 +20396,19 @@
       </c>
     </row>
     <row r="98" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A98" s="6" t="n">
+      <c r="A98" s="7" t="n">
         <v>46156</v>
       </c>
-      <c r="B98" s="3" t="n">
+      <c r="B98" s="5" t="n">
         <v>3746.3</v>
       </c>
-      <c r="C98" s="3" t="n">
+      <c r="C98" s="5" t="n">
         <v>5.53</v>
       </c>
-      <c r="D98" s="3" t="n">
+      <c r="D98" s="5" t="n">
         <v>2.27</v>
       </c>
-      <c r="E98" s="3" t="n">
+      <c r="E98" s="5" t="n">
         <v>10482.27</v>
       </c>
       <c r="F98" s="4" t="n">
@@ -20262,19 +20433,19 @@
       </c>
     </row>
     <row r="99" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A99" s="6" t="n">
+      <c r="A99" s="7" t="n">
         <v>46164</v>
       </c>
-      <c r="B99" s="3" t="n">
+      <c r="B99" s="5" t="n">
         <v>3849.9</v>
       </c>
-      <c r="C99" s="3" t="n">
+      <c r="C99" s="5" t="n">
         <v>5.62</v>
       </c>
-      <c r="D99" s="3" t="n">
+      <c r="D99" s="5" t="n">
         <v>2.31</v>
       </c>
-      <c r="E99" s="3" t="n">
+      <c r="E99" s="5" t="n">
         <v>10563.88</v>
       </c>
       <c r="F99" s="4" t="n">
@@ -20299,19 +20470,19 @@
       </c>
     </row>
     <row r="100" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A100" s="6" t="n">
+      <c r="A100" s="7" t="n">
         <v>46171</v>
       </c>
-      <c r="B100" s="3" t="n">
+      <c r="B100" s="5" t="n">
         <v>3880</v>
       </c>
-      <c r="C100" s="3" t="n">
+      <c r="C100" s="5" t="n">
         <v>5.53</v>
       </c>
-      <c r="D100" s="3" t="n">
+      <c r="D100" s="5" t="n">
         <v>2.38</v>
       </c>
-      <c r="E100" s="3" t="n">
+      <c r="E100" s="5" t="n">
         <v>10788.19</v>
       </c>
       <c r="F100" s="4" t="n">
@@ -20336,19 +20507,19 @@
       </c>
     </row>
     <row r="101" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A101" s="6" t="n">
+      <c r="A101" s="7" t="n">
         <v>46177</v>
       </c>
-      <c r="B101" s="3" t="n">
+      <c r="B101" s="5" t="n">
         <v>3600</v>
       </c>
-      <c r="C101" s="3" t="n">
+      <c r="C101" s="5" t="n">
         <v>5.57</v>
       </c>
-      <c r="D101" s="3" t="n">
+      <c r="D101" s="5" t="n">
         <v>2.45</v>
       </c>
-      <c r="E101" s="3" t="n">
+      <c r="E101" s="5" t="n">
         <v>10304.04</v>
       </c>
       <c r="F101" s="4" t="n">
@@ -20373,19 +20544,19 @@
       </c>
     </row>
     <row r="102" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A102" s="6" t="n">
+      <c r="A102" s="7" t="n">
         <v>46185</v>
       </c>
-      <c r="B102" s="3" t="n">
+      <c r="B102" s="5" t="n">
         <v>3712</v>
       </c>
-      <c r="C102" s="3" t="n">
+      <c r="C102" s="5" t="n">
         <v>5.54</v>
       </c>
-      <c r="D102" s="3" t="n">
+      <c r="D102" s="5" t="n">
         <v>2.5</v>
       </c>
-      <c r="E102" s="3" t="n">
+      <c r="E102" s="5" t="n">
         <v>10922.98</v>
       </c>
       <c r="F102" s="4" t="n">
@@ -20410,19 +20581,19 @@
       </c>
     </row>
     <row r="103" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A103" s="6" t="n">
+      <c r="A103" s="7" t="n">
         <v>46192</v>
       </c>
-      <c r="B103" s="3" t="n">
+      <c r="B103" s="5" t="n">
         <v>3820</v>
       </c>
-      <c r="C103" s="3" t="n">
+      <c r="C103" s="5" t="n">
         <v>5.45</v>
       </c>
-      <c r="D103" s="3" t="n">
+      <c r="D103" s="5" t="n">
         <v>2.49</v>
       </c>
-      <c r="E103" s="3" t="n">
+      <c r="E103" s="5" t="n">
         <v>10888.43</v>
       </c>
       <c r="F103" s="4" t="n">
@@ -20447,19 +20618,19 @@
       </c>
     </row>
     <row r="104" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A104" s="6" t="n">
+      <c r="A104" s="7" t="n">
         <v>46199</v>
       </c>
-      <c r="B104" s="3" t="n">
+      <c r="B104" s="5" t="n">
         <v>3765</v>
       </c>
-      <c r="C104" s="3" t="n">
+      <c r="C104" s="5" t="n">
         <v>5.45</v>
       </c>
-      <c r="D104" s="3" t="n">
+      <c r="D104" s="5" t="n">
         <v>2.43</v>
       </c>
-      <c r="E104" s="3" t="n">
+      <c r="E104" s="5" t="n">
         <v>10762.98</v>
       </c>
       <c r="F104" s="4" t="n">
@@ -20484,19 +20655,19 @@
       </c>
     </row>
     <row r="105" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A105" s="6" t="n">
+      <c r="A105" s="7" t="n">
         <v>46206</v>
       </c>
-      <c r="B105" s="3" t="n">
+      <c r="B105" s="5" t="n">
         <v>3919.7</v>
       </c>
-      <c r="C105" s="3" t="n">
+      <c r="C105" s="5" t="n">
         <v>5.42</v>
       </c>
-      <c r="D105" s="3" t="n">
+      <c r="D105" s="5" t="n">
         <v>2.45</v>
       </c>
-      <c r="E105" s="3" t="n">
+      <c r="E105" s="5" t="n">
         <v>10821.14</v>
       </c>
       <c r="F105" s="4" t="n">
@@ -20521,19 +20692,19 @@
       </c>
     </row>
     <row r="106" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A106" s="6" t="n">
+      <c r="A106" s="7" t="n">
         <v>46213</v>
       </c>
-      <c r="B106" s="3" t="n">
+      <c r="B106" s="5" t="n">
         <v>3901</v>
       </c>
-      <c r="C106" s="3" t="n">
+      <c r="C106" s="5" t="n">
         <v>5.48</v>
       </c>
-      <c r="D106" s="3" t="n">
+      <c r="D106" s="5" t="n">
         <v>2.42</v>
       </c>
-      <c r="E106" s="3" t="n">
+      <c r="E106" s="5" t="n">
         <v>10960.89</v>
       </c>
       <c r="F106" s="4" t="n">
@@ -20558,19 +20729,19 @@
       </c>
     </row>
     <row r="107" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A107" s="6" t="n">
+      <c r="A107" s="7" t="n">
         <v>46220</v>
       </c>
-      <c r="B107" s="3" t="n">
+      <c r="B107" s="5" t="n">
         <v>3950</v>
       </c>
-      <c r="C107" s="3" t="n">
+      <c r="C107" s="5" t="n">
         <v>5.54</v>
       </c>
-      <c r="D107" s="3" t="n">
+      <c r="D107" s="5" t="n">
         <v>2.44</v>
       </c>
-      <c r="E107" s="3" t="n">
+      <c r="E107" s="5" t="n">
         <v>10886.14</v>
       </c>
       <c r="F107" s="4" t="n">
@@ -20595,19 +20766,19 @@
       </c>
     </row>
     <row r="108" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A108" s="6" t="n">
+      <c r="A108" s="7" t="n">
         <v>46225</v>
       </c>
-      <c r="B108" s="3" t="n">
+      <c r="B108" s="5" t="n">
         <v>3820.2</v>
       </c>
-      <c r="C108" s="3" t="n">
+      <c r="C108" s="5" t="n">
         <v>5.68</v>
       </c>
-      <c r="D108" s="3" t="n">
+      <c r="D108" s="5" t="n">
         <v>2.48</v>
       </c>
-      <c r="E108" s="3" t="n">
+      <c r="E108" s="5" t="n">
         <v>11009.22</v>
       </c>
       <c r="F108" s="4" t="n">
@@ -20632,19 +20803,19 @@
       </c>
     </row>
     <row r="109" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A109" s="6" t="n">
+      <c r="A109" s="7" t="n">
         <v>46233</v>
       </c>
-      <c r="B109" s="3" t="n">
+      <c r="B109" s="5" t="n">
         <v>3690</v>
       </c>
-      <c r="C109" s="3" t="n">
+      <c r="C109" s="5" t="n">
         <v>5.68</v>
       </c>
-      <c r="D109" s="3" t="n">
+      <c r="D109" s="5" t="n">
         <v>2.53</v>
       </c>
-      <c r="E109" s="3" t="n">
+      <c r="E109" s="5" t="n">
         <v>11030.67</v>
       </c>
       <c r="F109" s="4" t="n">
@@ -20669,19 +20840,19 @@
       </c>
     </row>
     <row r="110" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A110" s="6" t="n">
+      <c r="A110" s="7" t="n">
         <v>46240</v>
       </c>
-      <c r="B110" s="3" t="n">
+      <c r="B110" s="5" t="n">
         <v>3940</v>
       </c>
-      <c r="C110" s="3" t="n">
+      <c r="C110" s="5" t="n">
         <v>5.63</v>
       </c>
-      <c r="D110" s="3" t="n">
+      <c r="D110" s="5" t="n">
         <v>2.56</v>
       </c>
-      <c r="E110" s="3" t="n">
+      <c r="E110" s="5" t="n">
         <v>11275.15</v>
       </c>
       <c r="F110" s="4" t="n">
@@ -20706,19 +20877,19 @@
       </c>
     </row>
     <row r="111" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A111" s="6" t="n">
+      <c r="A111" s="7" t="n">
         <v>46248</v>
       </c>
-      <c r="B111" s="3" t="n">
+      <c r="B111" s="5" t="n">
         <v>3970</v>
       </c>
-      <c r="C111" s="3" t="n">
+      <c r="C111" s="5" t="n">
         <v>5.66</v>
       </c>
-      <c r="D111" s="3" t="n">
+      <c r="D111" s="5" t="n">
         <v>2.52</v>
       </c>
-      <c r="E111" s="3" t="n">
+      <c r="E111" s="5" t="n">
         <v>11042.67</v>
       </c>
       <c r="F111" s="4" t="n">
@@ -20743,19 +20914,19 @@
       </c>
     </row>
     <row r="112" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A112" s="6" t="n">
+      <c r="A112" s="7" t="n">
         <v>46253</v>
       </c>
-      <c r="B112" s="3" t="n">
+      <c r="B112" s="5" t="n">
         <v>4000.1</v>
       </c>
-      <c r="C112" s="3" t="n">
+      <c r="C112" s="5" t="n">
         <v>5.7</v>
       </c>
-      <c r="D112" s="3" t="n">
+      <c r="D112" s="5" t="n">
         <v>2.51</v>
       </c>
-      <c r="E112" s="3" t="n">
+      <c r="E112" s="5" t="n">
         <v>11241.32</v>
       </c>
       <c r="F112" s="4" t="n">
@@ -20780,19 +20951,19 @@
       </c>
     </row>
     <row r="113" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A113" s="6" t="n">
+      <c r="A113" s="7" t="n">
         <v>46259</v>
       </c>
-      <c r="B113" s="3" t="n">
+      <c r="B113" s="5" t="n">
         <v>4062</v>
       </c>
-      <c r="C113" s="3" t="n">
+      <c r="C113" s="5" t="n">
         <v>5.7</v>
       </c>
-      <c r="D113" s="3" t="n">
+      <c r="D113" s="5" t="n">
         <v>2.51</v>
       </c>
-      <c r="E113" s="3" t="n">
+      <c r="E113" s="5" t="n">
         <v>11450.75</v>
       </c>
       <c r="F113" s="4" t="n">
@@ -20817,19 +20988,19 @@
       </c>
     </row>
     <row r="114" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A114" s="6" t="n">
+      <c r="A114" s="7" t="n">
         <v>46268</v>
       </c>
-      <c r="B114" s="3" t="n">
+      <c r="B114" s="5" t="n">
         <v>3955.04</v>
       </c>
-      <c r="C114" s="3" t="n">
+      <c r="C114" s="5" t="n">
         <v>5.71</v>
       </c>
-      <c r="D114" s="3" t="n">
+      <c r="D114" s="5" t="n">
         <v>2.54</v>
       </c>
-      <c r="E114" s="3" t="n">
+      <c r="E114" s="5" t="n">
         <v>11479.48</v>
       </c>
       <c r="F114" s="4" t="n">
@@ -20854,19 +21025,19 @@
       </c>
     </row>
     <row r="115" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A115" s="6" t="n">
+      <c r="A115" s="7" t="n">
         <v>46276</v>
       </c>
-      <c r="B115" s="3" t="n">
+      <c r="B115" s="5" t="n">
         <v>3850</v>
       </c>
-      <c r="C115" s="3" t="n">
+      <c r="C115" s="5" t="n">
         <v>6</v>
       </c>
-      <c r="D115" s="3" t="n">
+      <c r="D115" s="5" t="n">
         <v>2.52</v>
       </c>
-      <c r="E115" s="3" t="n">
+      <c r="E115" s="5" t="n">
         <v>11220.6</v>
       </c>
       <c r="F115" s="4" t="n">
@@ -20891,19 +21062,19 @@
       </c>
     </row>
     <row r="116" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A116" s="6" t="n">
+      <c r="A116" s="7" t="n">
         <v>46282</v>
       </c>
-      <c r="B116" s="3" t="n">
+      <c r="B116" s="5" t="n">
         <v>3900</v>
       </c>
-      <c r="C116" s="3" t="n">
+      <c r="C116" s="5" t="n">
         <v>6.03</v>
       </c>
-      <c r="D116" s="3" t="n">
+      <c r="D116" s="5" t="n">
         <v>2.62</v>
       </c>
-      <c r="E116" s="3" t="n">
+      <c r="E116" s="5" t="n">
         <v>11381.18</v>
       </c>
       <c r="F116" s="4" t="n">
@@ -20928,19 +21099,19 @@
       </c>
     </row>
     <row r="117" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A117" s="6" t="n">
+      <c r="A117" s="7" t="n">
         <v>46289</v>
       </c>
-      <c r="B117" s="3" t="n">
+      <c r="B117" s="5" t="n">
         <v>3666</v>
       </c>
-      <c r="C117" s="3" t="n">
+      <c r="C117" s="5" t="n">
         <v>6.04</v>
       </c>
-      <c r="D117" s="3" t="n">
+      <c r="D117" s="5" t="n">
         <v>2.73</v>
       </c>
-      <c r="E117" s="3" t="n">
+      <c r="E117" s="5" t="n">
         <v>11299.82</v>
       </c>
       <c r="F117" s="4" t="n">
@@ -20965,19 +21136,19 @@
       </c>
     </row>
     <row r="118" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A118" s="6" t="n">
+      <c r="A118" s="7" t="n">
         <v>46295</v>
       </c>
-      <c r="B118" s="3" t="n">
+      <c r="B118" s="5" t="n">
         <v>3555</v>
       </c>
-      <c r="C118" s="3" t="n">
+      <c r="C118" s="5" t="n">
         <v>6.25</v>
       </c>
-      <c r="D118" s="3" t="n">
+      <c r="D118" s="5" t="n">
         <v>2.82</v>
       </c>
-      <c r="E118" s="3" t="n">
+      <c r="E118" s="5" t="n">
         <v>10969.49</v>
       </c>
       <c r="F118" s="4" t="n">

</xml_diff>